<commit_message>
Cosmetici: TXT de importação com valores exatamente do XML (ICMS com diferimento, IPI, PIS, COFINS), auditoria campo a campo e IBS/CBS nas relações
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpFQAF7UfcTJUBPm398Z8s
</commit_message>
<xml_diff>
--- a/Cosmetici/Fiscal/2026-09/Relacao_Entradas_Cosmetici_09-2026.xlsx
+++ b/Cosmetici/Fiscal/2026-09/Relacao_Entradas_Cosmetici_09-2026.xlsx
@@ -15,8 +15,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas as entradas'!$A$4:$S$109</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NF-e dentro do estado (PR)'!$A$4:$AE$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NF-e fora do estado'!$A$4:$AE$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NF-e dentro do estado (PR)'!$A$4:$AH$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NF-e fora do estado'!$A$4:$AH$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CT-e'!$A$4:$R$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'NFS-e tomadas'!$A$4:$AA$25</definedName>
   </definedNames>
@@ -8009,7 +8009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE40"/>
+  <dimension ref="A1:AH40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8032,17 +8032,20 @@
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="8" customWidth="1" min="19" max="19"/>
     <col width="9" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="26" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="9" customWidth="1" min="25" max="25"/>
-    <col width="8" customWidth="1" min="26" max="26"/>
-    <col width="9" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="26" customWidth="1" min="29" max="29"/>
-    <col width="50" customWidth="1" min="30" max="30"/>
-    <col width="46" customWidth="1" min="31" max="31"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+    <col width="8" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="26" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="9" customWidth="1" min="28" max="28"/>
+    <col width="8" customWidth="1" min="29" max="29"/>
+    <col width="9" customWidth="1" min="30" max="30"/>
+    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="50" customWidth="1" min="33" max="33"/>
+    <col width="46" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8162,55 +8165,70 @@
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
+          <t>Base IBS/CBS</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>IBS</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>CBS</t>
+        </is>
+      </c>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
           <t>Total da nota</t>
         </is>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="Y4" s="3" t="inlineStr">
         <is>
           <t>Acumulador (sugestão)</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="Z4" s="3" t="inlineStr">
         <is>
           <t>Natureza</t>
         </is>
       </c>
-      <c r="X4" s="3" t="inlineStr">
+      <c r="AA4" s="3" t="inlineStr">
         <is>
           <t>Crédito ICMS</t>
         </is>
       </c>
-      <c r="Y4" s="3" t="inlineStr">
+      <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>Crédito IPI</t>
         </is>
       </c>
-      <c r="Z4" s="3" t="inlineStr">
+      <c r="AC4" s="3" t="inlineStr">
         <is>
           <t>DIFAL</t>
         </is>
       </c>
-      <c r="AA4" s="3" t="inlineStr">
+      <c r="AD4" s="3" t="inlineStr">
         <is>
           <t>ICMS antecipado</t>
         </is>
       </c>
-      <c r="AB4" s="3" t="inlineStr">
+      <c r="AE4" s="3" t="inlineStr">
         <is>
           <t>Conta contábil (Domínio)</t>
         </is>
       </c>
-      <c r="AC4" s="3" t="inlineStr">
+      <c r="AF4" s="3" t="inlineStr">
         <is>
           <t>Conferência XML x relatório SIEG</t>
         </is>
       </c>
-      <c r="AD4" s="3" t="inlineStr">
+      <c r="AG4" s="3" t="inlineStr">
         <is>
           <t>Análise</t>
         </is>
       </c>
-      <c r="AE4" s="3" t="inlineStr">
+      <c r="AH4" s="3" t="inlineStr">
         <is>
           <t>Chave de acesso</t>
         </is>
@@ -8294,44 +8312,53 @@
       <c r="U5" s="6" t="n">
         <v>3460</v>
       </c>
-      <c r="V5" s="5" t="inlineStr">
+      <c r="V5" s="6" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="W5" s="6" t="n">
+        <v>31.14</v>
+      </c>
+      <c r="X5" s="6" t="n">
+        <v>3460</v>
+      </c>
+      <c r="Y5" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">100 - COMPRA P/ INDUST - DENTRO </t>
         </is>
       </c>
-      <c r="W5" s="5" t="inlineStr">
+      <c r="Z5" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X5" s="6" t="n">
+      <c r="AA5" s="6" t="n">
         <v>98.95</v>
       </c>
-      <c r="Y5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="5" t="inlineStr">
+      <c r="AB5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC5" s="5" t="inlineStr">
+      <c r="AF5" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD5" s="5" t="inlineStr">
+      <c r="AG5" s="5" t="inlineStr">
         <is>
           <t>Simples CSOSN 101: crédito de 2.86% informado na nota (LC 123/06 art. 23 §1º)</t>
         </is>
       </c>
-      <c r="AE5" s="5" t="inlineStr">
+      <c r="AH5" s="5" t="inlineStr">
         <is>
           <t>41260906015875000143550010000037951000701710</t>
         </is>
@@ -8413,46 +8440,55 @@
         <v>125.06</v>
       </c>
       <c r="U6" s="6" t="n">
+        <v>1493.38</v>
+      </c>
+      <c r="V6" s="6" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="W6" s="6" t="n">
+        <v>13.44</v>
+      </c>
+      <c r="X6" s="6" t="n">
         <v>1870</v>
       </c>
-      <c r="V6" s="5" t="inlineStr">
+      <c r="Y6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">100 - COMPRA P/ INDUST - DENTRO </t>
         </is>
       </c>
-      <c r="W6" s="5" t="inlineStr">
+      <c r="Z6" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X6" s="6" t="n">
+      <c r="AA6" s="6" t="n">
         <v>224.41</v>
       </c>
-      <c r="Y6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="5" t="inlineStr">
+      <c r="AB6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506</t>
         </is>
       </c>
-      <c r="AC6" s="5" t="inlineStr">
+      <c r="AF6" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD6" s="5" t="inlineStr">
+      <c r="AG6" s="5" t="inlineStr">
         <is>
           <t>ICMS destacado (CST 51) em insumo (classificação do sped anterior)</t>
         </is>
       </c>
-      <c r="AE6" s="5" t="inlineStr">
+      <c r="AH6" s="5" t="inlineStr">
         <is>
           <t>41260904993269000177550010000417311010503945</t>
         </is>
@@ -8534,46 +8570,55 @@
         <v>0</v>
       </c>
       <c r="U7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="6" t="n">
         <v>2592</v>
       </c>
-      <c r="V7" s="5" t="inlineStr">
+      <c r="Y7" s="5" t="inlineStr">
         <is>
           <t>104 - COMPRA USO E CONSUMO DENTR</t>
         </is>
       </c>
-      <c r="W7" s="5" t="inlineStr">
+      <c r="Z7" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB7" s="5" t="inlineStr">
+      <c r="AB7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="5" t="inlineStr">
         <is>
           <t>D 513 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC7" s="5" t="inlineStr">
+      <c r="AF7" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD7" s="5" t="inlineStr">
+      <c r="AG7" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 102) - Uso e consumo (peça de manutenção): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE7" s="5" t="inlineStr">
+      <c r="AH7" s="5" t="inlineStr">
         <is>
           <t>41260966434370000145550010000003001634619321</t>
         </is>
@@ -8655,46 +8700,55 @@
         <v>0</v>
       </c>
       <c r="U8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="6" t="n">
         <v>3738</v>
       </c>
-      <c r="V8" s="5" t="inlineStr">
+      <c r="Y8" s="5" t="inlineStr">
         <is>
           <t>104 - COMPRA USO E CONSUMO DENTR</t>
         </is>
       </c>
-      <c r="W8" s="5" t="inlineStr">
+      <c r="Z8" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB8" s="5" t="inlineStr">
+      <c r="AB8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="5" t="inlineStr">
         <is>
           <t>D 513 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC8" s="5" t="inlineStr">
+      <c r="AF8" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD8" s="5" t="inlineStr">
+      <c r="AG8" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 101) - Uso e consumo (classificação do SPED anterior): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE8" s="5" t="inlineStr">
+      <c r="AH8" s="5" t="inlineStr">
         <is>
           <t>41260962341566000134550010000006951857187453</t>
         </is>
@@ -8776,46 +8830,55 @@
         <v>0</v>
       </c>
       <c r="U9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="6" t="n">
         <v>7052.79</v>
       </c>
-      <c r="V9" s="5" t="inlineStr">
+      <c r="Y9" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">100 - COMPRA P/ INDUST - DENTRO </t>
         </is>
       </c>
-      <c r="W9" s="5" t="inlineStr">
+      <c r="Z9" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z9" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB9" s="5" t="inlineStr">
+      <c r="AB9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="5" t="inlineStr">
         <is>
           <t>D 600 / C 506</t>
         </is>
       </c>
-      <c r="AC9" s="5" t="inlineStr">
+      <c r="AF9" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD9" s="5" t="inlineStr">
+      <c r="AG9" s="5" t="inlineStr">
         <is>
           <t>Simples CSOSN 102 (tributada SEM permissão de crédito): sem direito a crédito</t>
         </is>
       </c>
-      <c r="AE9" s="5" t="inlineStr">
+      <c r="AH9" s="5" t="inlineStr">
         <is>
           <t>41260952680145000184550010000007861702940405</t>
         </is>
@@ -8897,46 +8960,55 @@
         <v>0</v>
       </c>
       <c r="U10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="V10" s="5" t="inlineStr">
+      <c r="Y10" s="5" t="inlineStr">
         <is>
           <t>definir (CFOP 1923)</t>
         </is>
       </c>
-      <c r="W10" s="5" t="inlineStr">
+      <c r="Z10" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB10" s="5" t="inlineStr">
+      <c r="AB10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="5" t="inlineStr">
         <is>
           <t>sem conta: CFOP 1923 sem acumulador/conta no histórico do Domínio</t>
         </is>
       </c>
-      <c r="AC10" s="5" t="inlineStr">
+      <c r="AF10" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD10" s="5" t="inlineStr">
+      <c r="AG10" s="5" t="inlineStr">
         <is>
           <t>Remessa por conta e ordem de terceiros em venda à ordem (a venda vem em outra nota)</t>
         </is>
       </c>
-      <c r="AE10" s="5" t="inlineStr">
+      <c r="AH10" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000050271834583570</t>
         </is>
@@ -9018,46 +9090,55 @@
         <v>0</v>
       </c>
       <c r="U11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="V11" s="5" t="inlineStr">
+      <c r="Y11" s="5" t="inlineStr">
         <is>
           <t>155 - OUTRAS ENTRADAS DE MERCADO</t>
         </is>
       </c>
-      <c r="W11" s="5" t="inlineStr">
+      <c r="Z11" s="5" t="inlineStr">
         <is>
           <t>outras</t>
         </is>
       </c>
-      <c r="X11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z11" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB11" s="5" t="inlineStr">
+      <c r="AB11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" s="5" t="inlineStr">
         <is>
           <t>D 612 / C 613</t>
         </is>
       </c>
-      <c r="AC11" s="5" t="inlineStr">
+      <c r="AF11" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD11" s="5" t="inlineStr">
+      <c r="AG11" s="5" t="inlineStr">
         <is>
           <t>Matéria-prima (químico inorgânico) - mas CFOP 5949 (outras saídas: amostra/brinde/remessa): ICMS destacado R$ 0.20 não gera crédito</t>
         </is>
       </c>
-      <c r="AE11" s="5" t="inlineStr">
+      <c r="AH11" s="5" t="inlineStr">
         <is>
           <t>41260944114040000130550010000228371000945488</t>
         </is>
@@ -9139,46 +9220,55 @@
         <v>54.31</v>
       </c>
       <c r="U12" s="6" t="n">
+        <v>1744.1</v>
+      </c>
+      <c r="V12" s="6" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="W12" s="6" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="X12" s="6" t="n">
         <v>2248.65</v>
       </c>
-      <c r="V12" s="5" t="inlineStr">
+      <c r="Y12" s="5" t="inlineStr">
         <is>
           <t>104 - COMPRA USO E CONSUMO DENTR</t>
         </is>
       </c>
-      <c r="W12" s="5" t="inlineStr">
+      <c r="Z12" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA12" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB12" s="5" t="inlineStr">
+      <c r="AB12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="5" t="inlineStr">
         <is>
           <t>D 513 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC12" s="5" t="inlineStr">
+      <c r="AF12" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD12" s="5" t="inlineStr">
+      <c r="AG12" s="5" t="inlineStr">
         <is>
           <t>Uso e consumo (reagente de laboratório): ICMS destacado R$ 48.83 não gera crédito; Uso e consumo (reagente de laboratório): ICMS destacado R$ 43.40 não gera crédito; Uso e consumo (reagente de laboratório): ICMS destacado R$ 6.84 não gera crédito; Us</t>
         </is>
       </c>
-      <c r="AE12" s="5" t="inlineStr">
+      <c r="AH12" s="5" t="inlineStr">
         <is>
           <t>41260973636391000109550010001603261915612489</t>
         </is>
@@ -9260,46 +9350,55 @@
         <v>5.08</v>
       </c>
       <c r="U13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="6" t="n">
         <v>169.38</v>
       </c>
-      <c r="V13" s="5" t="inlineStr">
+      <c r="Y13" s="5" t="inlineStr">
         <is>
           <t>104 - COMPRA USO E CONSUMO DENTR</t>
         </is>
       </c>
-      <c r="W13" s="5" t="inlineStr">
+      <c r="Z13" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z13" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB13" s="5" t="inlineStr">
+      <c r="AB13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="5" t="inlineStr">
         <is>
           <t>D 513 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC13" s="5" t="inlineStr">
+      <c r="AF13" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD13" s="5" t="inlineStr">
+      <c r="AG13" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 102) - Uso e consumo (luva/artigo plástico): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE13" s="5" t="inlineStr">
+      <c r="AH13" s="5" t="inlineStr">
         <is>
           <t>41260941726398000125550010000049201009949200</t>
         </is>
@@ -9381,46 +9480,55 @@
         <v>0</v>
       </c>
       <c r="U14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="6" t="n">
         <v>1964</v>
       </c>
-      <c r="V14" s="5" t="inlineStr">
+      <c r="Y14" s="5" t="inlineStr">
         <is>
           <t>definir (CFOP 1923)</t>
         </is>
       </c>
-      <c r="W14" s="5" t="inlineStr">
+      <c r="Z14" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB14" s="5" t="inlineStr">
+      <c r="AB14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="5" t="inlineStr">
         <is>
           <t>sem conta: CFOP 1923 sem acumulador/conta no histórico do Domínio</t>
         </is>
       </c>
-      <c r="AC14" s="5" t="inlineStr">
+      <c r="AF14" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD14" s="5" t="inlineStr">
+      <c r="AG14" s="5" t="inlineStr">
         <is>
           <t>Remessa por conta e ordem de terceiros em venda à ordem (a venda vem em outra nota)</t>
         </is>
       </c>
-      <c r="AE14" s="5" t="inlineStr">
+      <c r="AH14" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000050481113690367</t>
         </is>
@@ -9498,30 +9606,39 @@
         <v>0</v>
       </c>
       <c r="U15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="12" t="n">
         <v>4370.44</v>
       </c>
-      <c r="V15" s="11" t="inlineStr">
+      <c r="Y15" s="11" t="inlineStr">
         <is>
           <t>cancelada (situação 02)</t>
         </is>
       </c>
-      <c r="W15" s="11" t="inlineStr"/>
-      <c r="X15" s="12" t="n"/>
-      <c r="Y15" s="12" t="n"/>
-      <c r="Z15" s="12" t="n"/>
+      <c r="Z15" s="11" t="inlineStr"/>
       <c r="AA15" s="12" t="n"/>
-      <c r="AB15" s="11" t="inlineStr">
+      <c r="AB15" s="12" t="n"/>
+      <c r="AC15" s="12" t="n"/>
+      <c r="AD15" s="12" t="n"/>
+      <c r="AE15" s="11" t="inlineStr">
         <is>
           <t>cancelada - sem lançamento</t>
         </is>
       </c>
-      <c r="AC15" s="11" t="inlineStr">
+      <c r="AF15" s="11" t="inlineStr">
         <is>
           <t>Cancelada - confere: evento de cancelamento no XML e status "Cancelamento" no relatório</t>
         </is>
       </c>
-      <c r="AD15" s="11" t="inlineStr"/>
-      <c r="AE15" s="11" t="inlineStr">
+      <c r="AG15" s="11" t="inlineStr"/>
+      <c r="AH15" s="11" t="inlineStr">
         <is>
           <t>41260952680145000184550010000007941049258979</t>
         </is>
@@ -9603,46 +9720,55 @@
         <v>0</v>
       </c>
       <c r="U16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="6" t="n">
         <v>4106.89</v>
       </c>
-      <c r="V16" s="5" t="inlineStr">
+      <c r="Y16" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">100 - COMPRA P/ INDUST - DENTRO </t>
         </is>
       </c>
-      <c r="W16" s="5" t="inlineStr">
+      <c r="Z16" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z16" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB16" s="5" t="inlineStr">
+      <c r="AB16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" s="5" t="inlineStr">
         <is>
           <t>D 600 / C 506</t>
         </is>
       </c>
-      <c r="AC16" s="5" t="inlineStr">
+      <c r="AF16" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD16" s="5" t="inlineStr">
+      <c r="AG16" s="5" t="inlineStr">
         <is>
           <t>Simples CSOSN 102 (tributada SEM permissão de crédito): sem direito a crédito</t>
         </is>
       </c>
-      <c r="AE16" s="5" t="inlineStr">
+      <c r="AH16" s="5" t="inlineStr">
         <is>
           <t>41260952680145000184550010000007951158784741</t>
         </is>
@@ -9724,46 +9850,55 @@
         <v>0</v>
       </c>
       <c r="U17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="6" t="n">
         <v>5670</v>
       </c>
-      <c r="V17" s="5" t="inlineStr">
+      <c r="Y17" s="5" t="inlineStr">
         <is>
           <t>165 - ENTRADA P/ IND POR CONTA E</t>
         </is>
       </c>
-      <c r="W17" s="5" t="inlineStr">
+      <c r="Z17" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z17" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB17" s="5" t="inlineStr">
+      <c r="AB17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="5" t="inlineStr">
         <is>
           <t>D 608 / C 609</t>
         </is>
       </c>
-      <c r="AC17" s="5" t="inlineStr">
+      <c r="AF17" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD17" s="5" t="inlineStr">
+      <c r="AG17" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por conta e ordem do adquirente (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE17" s="5" t="inlineStr">
+      <c r="AH17" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000050801135229929</t>
         </is>
@@ -9845,46 +9980,55 @@
         <v>0</v>
       </c>
       <c r="U18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" s="6" t="n">
         <v>2136</v>
       </c>
-      <c r="V18" s="5" t="inlineStr">
+      <c r="Y18" s="5" t="inlineStr">
         <is>
           <t>165 - ENTRADA P/ IND POR CONTA E</t>
         </is>
       </c>
-      <c r="W18" s="5" t="inlineStr">
+      <c r="Z18" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z18" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB18" s="5" t="inlineStr">
+      <c r="AB18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="5" t="inlineStr">
         <is>
           <t>D 608 / C 609</t>
         </is>
       </c>
-      <c r="AC18" s="5" t="inlineStr">
+      <c r="AF18" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD18" s="5" t="inlineStr">
+      <c r="AG18" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por conta e ordem do adquirente (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE18" s="5" t="inlineStr">
+      <c r="AH18" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000051331151580428</t>
         </is>
@@ -9966,46 +10110,55 @@
         <v>0</v>
       </c>
       <c r="U19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="6" t="n">
         <v>2286.82</v>
       </c>
-      <c r="V19" s="5" t="inlineStr">
+      <c r="Y19" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">100 - COMPRA P/ INDUST - DENTRO </t>
         </is>
       </c>
-      <c r="W19" s="5" t="inlineStr">
+      <c r="Z19" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB19" s="5" t="inlineStr">
+      <c r="AB19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="5" t="inlineStr">
         <is>
           <t>D 600 / C 506</t>
         </is>
       </c>
-      <c r="AC19" s="5" t="inlineStr">
+      <c r="AF19" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD19" s="5" t="inlineStr">
+      <c r="AG19" s="5" t="inlineStr">
         <is>
           <t>Simples CSOSN 102 (tributada SEM permissão de crédito): sem direito a crédito</t>
         </is>
       </c>
-      <c r="AE19" s="5" t="inlineStr">
+      <c r="AH19" s="5" t="inlineStr">
         <is>
           <t>41260937295717000118550010000137211931581334</t>
         </is>
@@ -10087,46 +10240,55 @@
         <v>0</v>
       </c>
       <c r="U20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" s="6" t="n">
         <v>1112</v>
       </c>
-      <c r="V20" s="5" t="inlineStr">
+      <c r="Y20" s="5" t="inlineStr">
         <is>
           <t>definir (CFOP 1923)</t>
         </is>
       </c>
-      <c r="W20" s="5" t="inlineStr">
+      <c r="Z20" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z20" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB20" s="5" t="inlineStr">
+      <c r="AB20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="5" t="inlineStr">
         <is>
           <t>sem conta: CFOP 1923 sem acumulador/conta no histórico do Domínio</t>
         </is>
       </c>
-      <c r="AC20" s="5" t="inlineStr">
+      <c r="AF20" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD20" s="5" t="inlineStr">
+      <c r="AG20" s="5" t="inlineStr">
         <is>
           <t>Remessa por conta e ordem de terceiros em venda à ordem (a venda vem em outra nota)</t>
         </is>
       </c>
-      <c r="AE20" s="5" t="inlineStr">
+      <c r="AH20" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000051621201311907</t>
         </is>
@@ -10208,46 +10370,55 @@
         <v>0</v>
       </c>
       <c r="U21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" s="6" t="n">
         <v>370.86</v>
       </c>
-      <c r="V21" s="5" t="inlineStr">
+      <c r="Y21" s="5" t="inlineStr">
         <is>
           <t>104 - COMPRA USO E CONSUMO DENTR</t>
         </is>
       </c>
-      <c r="W21" s="5" t="inlineStr">
+      <c r="Z21" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z21" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB21" s="5" t="inlineStr">
+      <c r="AB21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="5" t="inlineStr">
         <is>
           <t>D 656 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC21" s="5" t="inlineStr">
+      <c r="AF21" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD21" s="5" t="inlineStr">
+      <c r="AG21" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 102) - Uso e consumo (classificação do SPED anterior): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE21" s="5" t="inlineStr">
+      <c r="AH21" s="5" t="inlineStr">
         <is>
           <t>41260910265455000192550010000404511000405060</t>
         </is>
@@ -10331,44 +10502,53 @@
       <c r="U22" s="6" t="n">
         <v>1320.74</v>
       </c>
-      <c r="V22" s="5" t="inlineStr">
+      <c r="V22" s="6" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="W22" s="6" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="X22" s="6" t="n">
+        <v>1320.74</v>
+      </c>
+      <c r="Y22" s="5" t="inlineStr">
         <is>
           <t>104 - COMPRA USO E CONSUMO DENTR</t>
         </is>
       </c>
-      <c r="W22" s="5" t="inlineStr">
+      <c r="Z22" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA22" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB22" s="5" t="inlineStr">
+      <c r="AB22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="5" t="inlineStr">
         <is>
           <t>D 513 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC22" s="5" t="inlineStr">
+      <c r="AF22" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD22" s="5" t="inlineStr">
+      <c r="AG22" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 103) - Uso e consumo (classificação do SPED anterior): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE22" s="5" t="inlineStr">
+      <c r="AH22" s="5" t="inlineStr">
         <is>
           <t>41260959087034000108550010000004181258202600</t>
         </is>
@@ -10450,46 +10630,55 @@
         <v>0</v>
       </c>
       <c r="U23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" s="6" t="n">
         <v>667.2</v>
       </c>
-      <c r="V23" s="5" t="inlineStr">
+      <c r="Y23" s="5" t="inlineStr">
         <is>
           <t>165 - ENTRADA P/ IND POR CONTA E</t>
         </is>
       </c>
-      <c r="W23" s="5" t="inlineStr">
+      <c r="Z23" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z23" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA23" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB23" s="5" t="inlineStr">
+      <c r="AB23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="5" t="inlineStr">
         <is>
           <t>D 608 / C 609</t>
         </is>
       </c>
-      <c r="AC23" s="5" t="inlineStr">
+      <c r="AF23" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD23" s="5" t="inlineStr">
+      <c r="AG23" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por conta e ordem do adquirente (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE23" s="5" t="inlineStr">
+      <c r="AH23" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000051701177572396</t>
         </is>
@@ -10571,46 +10760,55 @@
         <v>0</v>
       </c>
       <c r="U24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" s="6" t="n">
         <v>273.5</v>
       </c>
-      <c r="V24" s="5" t="inlineStr">
+      <c r="Y24" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">100 - COMPRA P/ INDUST - DENTRO </t>
         </is>
       </c>
-      <c r="W24" s="5" t="inlineStr">
+      <c r="Z24" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z24" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA24" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB24" s="5" t="inlineStr">
+      <c r="AB24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="5" t="inlineStr">
         <is>
           <t>D 600 / C 506</t>
         </is>
       </c>
-      <c r="AC24" s="5" t="inlineStr">
+      <c r="AF24" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD24" s="5" t="inlineStr">
+      <c r="AG24" s="5" t="inlineStr">
         <is>
           <t>Simples CSOSN 102 (tributada SEM permissão de crédito): sem direito a crédito</t>
         </is>
       </c>
-      <c r="AE24" s="5" t="inlineStr">
+      <c r="AH24" s="5" t="inlineStr">
         <is>
           <t>41260952680145000184550010000008141610067850</t>
         </is>
@@ -10692,46 +10890,55 @@
         <v>55.57</v>
       </c>
       <c r="U25" s="6" t="n">
+        <v>731.21</v>
+      </c>
+      <c r="V25" s="6" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="W25" s="6" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="X25" s="6" t="n">
         <v>833.9</v>
       </c>
-      <c r="V25" s="5" t="inlineStr">
+      <c r="Y25" s="5" t="inlineStr">
         <is>
           <t>104 - COMPRA USO E CONSUMO DENTR</t>
         </is>
       </c>
-      <c r="W25" s="5" t="inlineStr">
+      <c r="Z25" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X25" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y25" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z25" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA25" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB25" s="5" t="inlineStr">
+      <c r="AB25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" s="5" t="inlineStr">
         <is>
           <t>D 513 / C 506</t>
         </is>
       </c>
-      <c r="AC25" s="5" t="inlineStr">
+      <c r="AF25" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD25" s="5" t="inlineStr">
+      <c r="AG25" s="5" t="inlineStr">
         <is>
           <t>Uso e consumo (pano/TNT/EPI): ICMS destacado R$ 95.88 não gera crédito; Uso e consumo (ferramenta/limpeza): ICMS destacado R$ 6.81 não gera crédito</t>
         </is>
       </c>
-      <c r="AE25" s="5" t="inlineStr">
+      <c r="AH25" s="5" t="inlineStr">
         <is>
           <t>41260949547438000183550010000067821963905200</t>
         </is>
@@ -10813,46 +11020,55 @@
         <v>0</v>
       </c>
       <c r="U26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X26" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="V26" s="5" t="inlineStr">
+      <c r="Y26" s="5" t="inlineStr">
         <is>
           <t>155 - OUTRAS ENTRADAS DE MERCADO</t>
         </is>
       </c>
-      <c r="W26" s="5" t="inlineStr">
+      <c r="Z26" s="5" t="inlineStr">
         <is>
           <t>outras</t>
         </is>
       </c>
-      <c r="X26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z26" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA26" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB26" s="5" t="inlineStr">
+      <c r="AB26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE26" s="5" t="inlineStr">
         <is>
           <t>D 612 / C 613</t>
         </is>
       </c>
-      <c r="AC26" s="5" t="inlineStr">
+      <c r="AF26" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD26" s="5" t="inlineStr">
+      <c r="AG26" s="5" t="inlineStr">
         <is>
           <t>Matéria-prima (químico orgânico) - mas CFOP 5949 (outras saídas: amostra/brinde/remessa): ICMS destacado R$ 0.20 não gera crédito</t>
         </is>
       </c>
-      <c r="AE26" s="5" t="inlineStr">
+      <c r="AH26" s="5" t="inlineStr">
         <is>
           <t>41260944114040000130550010000231271000948452</t>
         </is>
@@ -10936,44 +11152,53 @@
       <c r="U27" s="6" t="n">
         <v>1140</v>
       </c>
-      <c r="V27" s="5" t="inlineStr">
+      <c r="V27" s="6" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="W27" s="6" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="X27" s="6" t="n">
+        <v>1140</v>
+      </c>
+      <c r="Y27" s="5" t="inlineStr">
         <is>
           <t>104 - COMPRA USO E CONSUMO DENTR</t>
         </is>
       </c>
-      <c r="W27" s="5" t="inlineStr">
+      <c r="Z27" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z27" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA27" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB27" s="5" t="inlineStr">
+      <c r="AB27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE27" s="5" t="inlineStr">
         <is>
           <t>D 513 / C 506</t>
         </is>
       </c>
-      <c r="AC27" s="5" t="inlineStr">
+      <c r="AF27" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD27" s="5" t="inlineStr">
+      <c r="AG27" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 103) - Uso e consumo (classificação do SPED anterior): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE27" s="5" t="inlineStr">
+      <c r="AH27" s="5" t="inlineStr">
         <is>
           <t>41260925141658000144550020000032141236266620</t>
         </is>
@@ -11055,46 +11280,55 @@
         <v>0</v>
       </c>
       <c r="U28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" s="6" t="n">
         <v>5700</v>
       </c>
-      <c r="V28" s="5" t="inlineStr">
+      <c r="Y28" s="5" t="inlineStr">
         <is>
           <t>149 - ENTRADA PARA IND. POR ENCO</t>
         </is>
       </c>
-      <c r="W28" s="5" t="inlineStr">
+      <c r="Z28" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X28" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y28" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z28" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA28" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB28" s="5" t="inlineStr">
+      <c r="AB28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="5" t="inlineStr">
         <is>
           <t>D 614 / C 607</t>
         </is>
       </c>
-      <c r="AC28" s="5" t="inlineStr">
+      <c r="AF28" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD28" s="5" t="inlineStr">
+      <c r="AG28" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 400) - Remessa para industrialização por encomenda (insumo do cliente): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE28" s="5" t="inlineStr">
+      <c r="AH28" s="5" t="inlineStr">
         <is>
           <t>41260918074269000188550010000171871932036922</t>
         </is>
@@ -11176,46 +11410,55 @@
         <v>0</v>
       </c>
       <c r="U29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X29" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="V29" s="5" t="inlineStr">
+      <c r="Y29" s="5" t="inlineStr">
         <is>
           <t>149 - ENTRADA PARA IND. POR ENCO</t>
         </is>
       </c>
-      <c r="W29" s="5" t="inlineStr">
+      <c r="Z29" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z29" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA29" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB29" s="5" t="inlineStr">
+      <c r="AB29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="5" t="inlineStr">
         <is>
           <t>D 614 / C 607</t>
         </is>
       </c>
-      <c r="AC29" s="5" t="inlineStr">
+      <c r="AF29" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD29" s="5" t="inlineStr">
+      <c r="AG29" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 500) - Remessa para industrialização por encomenda (insumo do cliente): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE29" s="5" t="inlineStr">
+      <c r="AH29" s="5" t="inlineStr">
         <is>
           <t>41260921822008000103550020000045511028307079</t>
         </is>
@@ -11297,46 +11540,55 @@
         <v>0</v>
       </c>
       <c r="U30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" s="6" t="n">
         <v>2420.01</v>
       </c>
-      <c r="V30" s="5" t="inlineStr">
+      <c r="Y30" s="5" t="inlineStr">
         <is>
           <t>165 - ENTRADA P/ IND POR CONTA E</t>
         </is>
       </c>
-      <c r="W30" s="5" t="inlineStr">
+      <c r="Z30" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z30" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA30" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB30" s="5" t="inlineStr">
+      <c r="AB30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE30" s="5" t="inlineStr">
         <is>
           <t>D 608 / C 609</t>
         </is>
       </c>
-      <c r="AC30" s="5" t="inlineStr">
+      <c r="AF30" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD30" s="5" t="inlineStr">
+      <c r="AG30" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por conta e ordem do adquirente (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE30" s="5" t="inlineStr">
+      <c r="AH30" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000052331135756040</t>
         </is>
@@ -11418,46 +11670,55 @@
         <v>0</v>
       </c>
       <c r="U31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X31" s="6" t="n">
         <v>1760</v>
       </c>
-      <c r="V31" s="5" t="inlineStr">
+      <c r="Y31" s="5" t="inlineStr">
         <is>
           <t>165 - ENTRADA P/ IND POR CONTA E</t>
         </is>
       </c>
-      <c r="W31" s="5" t="inlineStr">
+      <c r="Z31" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X31" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y31" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z31" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB31" s="5" t="inlineStr">
+      <c r="AB31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE31" s="5" t="inlineStr">
         <is>
           <t>D 608 / C 609</t>
         </is>
       </c>
-      <c r="AC31" s="5" t="inlineStr">
+      <c r="AF31" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD31" s="5" t="inlineStr">
+      <c r="AG31" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por conta e ordem do adquirente (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE31" s="5" t="inlineStr">
+      <c r="AH31" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000052351191452986</t>
         </is>
@@ -11539,46 +11800,55 @@
         <v>0</v>
       </c>
       <c r="U32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="V32" s="5" t="inlineStr">
+      <c r="Y32" s="5" t="inlineStr">
         <is>
           <t>149 - ENTRADA PARA IND. POR ENCO</t>
         </is>
       </c>
-      <c r="W32" s="5" t="inlineStr">
+      <c r="Z32" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X32" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y32" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z32" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA32" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB32" s="5" t="inlineStr">
+      <c r="AB32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE32" s="5" t="inlineStr">
         <is>
           <t>D 614 / C 607</t>
         </is>
       </c>
-      <c r="AC32" s="5" t="inlineStr">
+      <c r="AF32" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD32" s="5" t="inlineStr">
+      <c r="AG32" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por encomenda (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE32" s="5" t="inlineStr">
+      <c r="AH32" s="5" t="inlineStr">
         <is>
           <t>41260906237330000181550010000558741118273450</t>
         </is>
@@ -11660,46 +11930,55 @@
         <v>0</v>
       </c>
       <c r="U33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X33" s="6" t="n">
         <v>556.5</v>
       </c>
-      <c r="V33" s="5" t="inlineStr">
+      <c r="Y33" s="5" t="inlineStr">
         <is>
           <t>149 - ENTRADA PARA IND. POR ENCO</t>
         </is>
       </c>
-      <c r="W33" s="5" t="inlineStr">
+      <c r="Z33" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X33" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y33" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z33" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB33" s="5" t="inlineStr">
+      <c r="AB33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE33" s="5" t="inlineStr">
         <is>
           <t>D 614 / C 607</t>
         </is>
       </c>
-      <c r="AC33" s="5" t="inlineStr">
+      <c r="AF33" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD33" s="5" t="inlineStr">
+      <c r="AG33" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por encomenda (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE33" s="5" t="inlineStr">
+      <c r="AH33" s="5" t="inlineStr">
         <is>
           <t>41260906237330000181550010000559131118294105</t>
         </is>
@@ -11781,46 +12060,55 @@
         <v>0</v>
       </c>
       <c r="U34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X34" s="6" t="n">
         <v>1893</v>
       </c>
-      <c r="V34" s="5" t="inlineStr">
+      <c r="Y34" s="5" t="inlineStr">
         <is>
           <t>155 - OUTRAS ENTRADAS DE MERCADO</t>
         </is>
       </c>
-      <c r="W34" s="5" t="inlineStr">
+      <c r="Z34" s="5" t="inlineStr">
         <is>
           <t>outras</t>
         </is>
       </c>
-      <c r="X34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z34" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA34" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB34" s="5" t="inlineStr">
+      <c r="AB34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE34" s="5" t="inlineStr">
         <is>
           <t>D 612 / C 613</t>
         </is>
       </c>
-      <c r="AC34" s="5" t="inlineStr">
+      <c r="AF34" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD34" s="5" t="inlineStr">
+      <c r="AG34" s="5" t="inlineStr">
         <is>
           <t>Embalagem (rótulo/etiqueta) - mas CFOP 5949 (outras saídas: amostra/brinde/remessa)</t>
         </is>
       </c>
-      <c r="AE34" s="5" t="inlineStr">
+      <c r="AH34" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000053821102007626</t>
         </is>
@@ -11902,46 +12190,55 @@
         <v>0</v>
       </c>
       <c r="U35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="V35" s="5" t="inlineStr">
+      <c r="Y35" s="5" t="inlineStr">
         <is>
           <t>149 - ENTRADA PARA IND. POR ENCO</t>
         </is>
       </c>
-      <c r="W35" s="5" t="inlineStr">
+      <c r="Z35" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X35" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y35" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z35" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA35" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB35" s="5" t="inlineStr">
+      <c r="AB35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE35" s="5" t="inlineStr">
         <is>
           <t>D 614 / C 607</t>
         </is>
       </c>
-      <c r="AC35" s="5" t="inlineStr">
+      <c r="AF35" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD35" s="5" t="inlineStr">
+      <c r="AG35" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por encomenda (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE35" s="5" t="inlineStr">
+      <c r="AH35" s="5" t="inlineStr">
         <is>
           <t>41260906237330000181550010000560041118322920</t>
         </is>
@@ -12023,46 +12320,55 @@
         <v>0</v>
       </c>
       <c r="U36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X36" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="V36" s="5" t="inlineStr">
+      <c r="Y36" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">100 - COMPRA P/ INDUST - DENTRO </t>
         </is>
       </c>
-      <c r="W36" s="5" t="inlineStr">
+      <c r="Z36" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X36" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y36" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z36" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA36" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB36" s="5" t="inlineStr">
+      <c r="AB36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE36" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506</t>
         </is>
       </c>
-      <c r="AC36" s="5" t="inlineStr">
+      <c r="AF36" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD36" s="5" t="inlineStr">
+      <c r="AG36" s="5" t="inlineStr">
         <is>
           <t>Simples CSOSN 102 (tributada SEM permissão de crédito): sem direito a crédito</t>
         </is>
       </c>
-      <c r="AE36" s="5" t="inlineStr">
+      <c r="AH36" s="5" t="inlineStr">
         <is>
           <t>41260976509488000149550010002220981017634246</t>
         </is>
@@ -12144,46 +12450,55 @@
         <v>0</v>
       </c>
       <c r="U37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" s="6" t="n">
         <v>1180</v>
       </c>
-      <c r="V37" s="5" t="inlineStr">
+      <c r="Y37" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">100 - COMPRA P/ INDUST - DENTRO </t>
         </is>
       </c>
-      <c r="W37" s="5" t="inlineStr">
+      <c r="Z37" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z37" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA37" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB37" s="5" t="inlineStr">
+      <c r="AB37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE37" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC37" s="5" t="inlineStr">
+      <c r="AF37" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD37" s="5" t="inlineStr">
+      <c r="AG37" s="5" t="inlineStr">
         <is>
           <t>Simples CSOSN 101 sem percentual de crédito (pCredSN 0%); Sem crédito: segue o XML (CSOSN com permissão de crédito, mas sem % informado)</t>
         </is>
       </c>
-      <c r="AE37" s="5" t="inlineStr">
+      <c r="AH37" s="5" t="inlineStr">
         <is>
           <t>41260963460684000124550010000000421742919846</t>
         </is>
@@ -12265,46 +12580,55 @@
         <v>374.09</v>
       </c>
       <c r="U38" s="6" t="n">
+        <v>4466.97</v>
+      </c>
+      <c r="V38" s="6" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="W38" s="6" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="X38" s="6" t="n">
         <v>5593.5</v>
       </c>
-      <c r="V38" s="5" t="inlineStr">
+      <c r="Y38" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">100 - COMPRA P/ INDUST - DENTRO </t>
         </is>
       </c>
-      <c r="W38" s="5" t="inlineStr">
+      <c r="Z38" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X38" s="6" t="n">
+      <c r="AA38" s="6" t="n">
         <v>671.22</v>
       </c>
-      <c r="Y38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB38" s="5" t="inlineStr">
+      <c r="AB38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE38" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506</t>
         </is>
       </c>
-      <c r="AC38" s="5" t="inlineStr">
+      <c r="AF38" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD38" s="5" t="inlineStr">
+      <c r="AG38" s="5" t="inlineStr">
         <is>
           <t>ICMS destacado (CST 51) em insumo (classificação do sped anterior)</t>
         </is>
       </c>
-      <c r="AE38" s="5" t="inlineStr">
+      <c r="AH38" s="5" t="inlineStr">
         <is>
           <t>41260916987597000140550010000381751288422874</t>
         </is>
@@ -12386,46 +12710,55 @@
         <v>3.53</v>
       </c>
       <c r="U39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" s="6" t="n">
         <v>389.77</v>
       </c>
-      <c r="V39" s="5" t="inlineStr">
+      <c r="Y39" s="5" t="inlineStr">
         <is>
           <t>104 - COMPRA USO E CONSUMO DENTR</t>
         </is>
       </c>
-      <c r="W39" s="5" t="inlineStr">
+      <c r="Z39" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X39" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y39" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z39" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA39" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB39" s="5" t="inlineStr">
+      <c r="AB39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE39" s="5" t="inlineStr">
         <is>
           <t>D 360 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC39" s="5" t="inlineStr">
+      <c r="AF39" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD39" s="5" t="inlineStr">
+      <c r="AG39" s="5" t="inlineStr">
         <is>
           <t>Uso e consumo (classificação do SPED anterior); Uso e consumo (classificação do SPED anterior): ICMS destacado R$ 5.40 não gera crédito</t>
         </is>
       </c>
-      <c r="AE39" s="5" t="inlineStr">
+      <c r="AH39" s="5" t="inlineStr">
         <is>
           <t>41260973419905000174550010000971451002693820</t>
         </is>
@@ -12496,31 +12829,43 @@
         <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*U5:U39)</f>
         <v/>
       </c>
-      <c r="V40" s="17" t="n"/>
-      <c r="W40" s="17" t="n"/>
+      <c r="V40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*V5:V39)</f>
+        <v/>
+      </c>
+      <c r="W40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*W5:W39)</f>
+        <v/>
+      </c>
       <c r="X40" s="18">
         <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*X5:X39)</f>
         <v/>
       </c>
-      <c r="Y40" s="18">
-        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*Y5:Y39)</f>
-        <v/>
-      </c>
-      <c r="Z40" s="18">
-        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*Z5:Z39)</f>
-        <v/>
-      </c>
+      <c r="Y40" s="17" t="n"/>
+      <c r="Z40" s="17" t="n"/>
       <c r="AA40" s="18">
         <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*AA5:AA39)</f>
         <v/>
       </c>
-      <c r="AB40" s="17" t="n"/>
-      <c r="AC40" s="17" t="n"/>
-      <c r="AD40" s="17" t="n"/>
+      <c r="AB40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*AB5:AB39)</f>
+        <v/>
+      </c>
+      <c r="AC40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*AC5:AC39)</f>
+        <v/>
+      </c>
+      <c r="AD40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*AD5:AD39)</f>
+        <v/>
+      </c>
       <c r="AE40" s="17" t="n"/>
+      <c r="AF40" s="17" t="n"/>
+      <c r="AG40" s="17" t="n"/>
+      <c r="AH40" s="17" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AE39"/>
+  <autoFilter ref="A4:AH39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -12532,7 +12877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE24"/>
+  <dimension ref="A1:AH24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12555,17 +12900,20 @@
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="8" customWidth="1" min="19" max="19"/>
     <col width="9" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="26" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="9" customWidth="1" min="25" max="25"/>
-    <col width="8" customWidth="1" min="26" max="26"/>
-    <col width="9" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="26" customWidth="1" min="29" max="29"/>
-    <col width="50" customWidth="1" min="30" max="30"/>
-    <col width="46" customWidth="1" min="31" max="31"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+    <col width="8" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="26" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="9" customWidth="1" min="28" max="28"/>
+    <col width="8" customWidth="1" min="29" max="29"/>
+    <col width="9" customWidth="1" min="30" max="30"/>
+    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="50" customWidth="1" min="33" max="33"/>
+    <col width="46" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12685,55 +13033,70 @@
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
+          <t>Base IBS/CBS</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>IBS</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>CBS</t>
+        </is>
+      </c>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
           <t>Total da nota</t>
         </is>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="Y4" s="3" t="inlineStr">
         <is>
           <t>Acumulador (sugestão)</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="Z4" s="3" t="inlineStr">
         <is>
           <t>Natureza</t>
         </is>
       </c>
-      <c r="X4" s="3" t="inlineStr">
+      <c r="AA4" s="3" t="inlineStr">
         <is>
           <t>Crédito ICMS</t>
         </is>
       </c>
-      <c r="Y4" s="3" t="inlineStr">
+      <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>Crédito IPI</t>
         </is>
       </c>
-      <c r="Z4" s="3" t="inlineStr">
+      <c r="AC4" s="3" t="inlineStr">
         <is>
           <t>DIFAL</t>
         </is>
       </c>
-      <c r="AA4" s="3" t="inlineStr">
+      <c r="AD4" s="3" t="inlineStr">
         <is>
           <t>ICMS antecipado</t>
         </is>
       </c>
-      <c r="AB4" s="3" t="inlineStr">
+      <c r="AE4" s="3" t="inlineStr">
         <is>
           <t>Conta contábil (Domínio)</t>
         </is>
       </c>
-      <c r="AC4" s="3" t="inlineStr">
+      <c r="AF4" s="3" t="inlineStr">
         <is>
           <t>Conferência XML x relatório SIEG</t>
         </is>
       </c>
-      <c r="AD4" s="3" t="inlineStr">
+      <c r="AG4" s="3" t="inlineStr">
         <is>
           <t>Análise</t>
         </is>
       </c>
-      <c r="AE4" s="3" t="inlineStr">
+      <c r="AH4" s="3" t="inlineStr">
         <is>
           <t>Chave de acesso</t>
         </is>
@@ -12815,46 +13178,55 @@
         <v>0</v>
       </c>
       <c r="U5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="6" t="n">
         <v>924</v>
       </c>
-      <c r="V5" s="5" t="inlineStr">
+      <c r="Y5" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">105 - COMPRA USO E CONSUMO FORA </t>
         </is>
       </c>
-      <c r="W5" s="5" t="inlineStr">
+      <c r="Z5" s="5" t="inlineStr">
         <is>
           <t>uso</t>
         </is>
       </c>
-      <c r="X5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="6" t="n">
+      <c r="AA5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="6" t="n">
         <v>86.09</v>
       </c>
-      <c r="AA5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="5" t="inlineStr">
+      <c r="AD5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="5" t="inlineStr">
         <is>
           <t>D 513 / C 506</t>
         </is>
       </c>
-      <c r="AC5" s="5" t="inlineStr">
+      <c r="AF5" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD5" s="5" t="inlineStr">
+      <c r="AG5" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 201) - Uso e consumo (classificação do SPED anterior): sem crédito (só mercadoria para industrialização/comercialização); DIFAL R$ 86.09 (base dupla) - ajuste a débito PR000081</t>
         </is>
       </c>
-      <c r="AE5" s="5" t="inlineStr">
+      <c r="AH5" s="5" t="inlineStr">
         <is>
           <t>43260954079636000108550010000025641087230517</t>
         </is>
@@ -12936,46 +13308,55 @@
         <v>0</v>
       </c>
       <c r="U6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="6" t="n">
         <v>1408.12</v>
       </c>
-      <c r="V6" s="5" t="inlineStr">
+      <c r="Y6" s="5" t="inlineStr">
         <is>
           <t>164 - ENTRADA P/ IND POR CONTA E</t>
         </is>
       </c>
-      <c r="W6" s="5" t="inlineStr">
+      <c r="Z6" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB6" s="5" t="inlineStr">
+      <c r="AB6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="5" t="inlineStr">
         <is>
           <t>D 608 / C 609</t>
         </is>
       </c>
-      <c r="AC6" s="5" t="inlineStr">
+      <c r="AF6" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD6" s="5" t="inlineStr">
+      <c r="AG6" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 101) - Remessa para industrialização por conta e ordem do adquirente (insumo do cliente): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE6" s="5" t="inlineStr">
+      <c r="AH6" s="5" t="inlineStr">
         <is>
           <t>35260939237959000180550010000080991000082318</t>
         </is>
@@ -13057,46 +13438,55 @@
         <v>0</v>
       </c>
       <c r="U7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="6" t="n">
         <v>2462.03</v>
       </c>
-      <c r="V7" s="5" t="inlineStr">
+      <c r="Y7" s="5" t="inlineStr">
         <is>
           <t>164 - ENTRADA P/ IND POR CONTA E</t>
         </is>
       </c>
-      <c r="W7" s="5" t="inlineStr">
+      <c r="Z7" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB7" s="5" t="inlineStr">
+      <c r="AB7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="5" t="inlineStr">
         <is>
           <t>D 608 / C 609</t>
         </is>
       </c>
-      <c r="AC7" s="5" t="inlineStr">
+      <c r="AF7" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD7" s="5" t="inlineStr">
+      <c r="AG7" s="5" t="inlineStr">
         <is>
           <t>Simples (CSOSN 101) - Remessa para industrialização por conta e ordem do adquirente (insumo do cliente): sem crédito (só mercadoria para industrialização/comercialização)</t>
         </is>
       </c>
-      <c r="AE7" s="5" t="inlineStr">
+      <c r="AH7" s="5" t="inlineStr">
         <is>
           <t>35260934970658000148550010000081121000087609</t>
         </is>
@@ -13178,46 +13568,55 @@
         <v>66.17</v>
       </c>
       <c r="U8" s="6" t="n">
+        <v>2426.05</v>
+      </c>
+      <c r="V8" s="6" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="W8" s="6" t="n">
+        <v>21.83</v>
+      </c>
+      <c r="X8" s="6" t="n">
         <v>2506.56</v>
       </c>
-      <c r="V8" s="5" t="inlineStr">
+      <c r="Y8" s="5" t="inlineStr">
         <is>
           <t>101 - COMPRA P/ INDUST - FORA ES</t>
         </is>
       </c>
-      <c r="W8" s="5" t="inlineStr">
+      <c r="Z8" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X8" s="6" t="n">
+      <c r="AA8" s="6" t="n">
         <v>300.79</v>
       </c>
-      <c r="Y8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="5" t="inlineStr">
+      <c r="AB8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC8" s="5" t="inlineStr">
+      <c r="AF8" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD8" s="5" t="inlineStr">
+      <c r="AG8" s="5" t="inlineStr">
         <is>
           <t>ICMS destacado (CST 00) em embalagem (tampa metálica)</t>
         </is>
       </c>
-      <c r="AE8" s="5" t="inlineStr">
+      <c r="AH8" s="5" t="inlineStr">
         <is>
           <t>35260967598292000187550010000303381000323387</t>
         </is>
@@ -13299,46 +13698,55 @@
         <v>1665.12</v>
       </c>
       <c r="U9" s="6" t="n">
+        <v>19882.89</v>
+      </c>
+      <c r="V9" s="6" t="n">
+        <v>19.88</v>
+      </c>
+      <c r="W9" s="6" t="n">
+        <v>178.95</v>
+      </c>
+      <c r="X9" s="6" t="n">
         <v>26515.5</v>
       </c>
-      <c r="V9" s="5" t="inlineStr">
+      <c r="Y9" s="5" t="inlineStr">
         <is>
           <t>101 - COMPRA P/ INDUST - FORA ES</t>
         </is>
       </c>
-      <c r="W9" s="5" t="inlineStr">
+      <c r="Z9" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X9" s="6" t="n">
+      <c r="AA9" s="6" t="n">
         <v>2987.66</v>
       </c>
-      <c r="Y9" s="6" t="n">
+      <c r="AB9" s="6" t="n">
         <v>1618.32</v>
       </c>
-      <c r="Z9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB9" s="5" t="inlineStr">
+      <c r="AC9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506 (conferir)</t>
         </is>
       </c>
-      <c r="AC9" s="5" t="inlineStr">
+      <c r="AF9" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD9" s="5" t="inlineStr">
+      <c r="AG9" s="5" t="inlineStr">
         <is>
           <t>ICMS destacado (CST 00) em embalagem (tubo de alumínio)</t>
         </is>
       </c>
-      <c r="AE9" s="5" t="inlineStr">
+      <c r="AH9" s="5" t="inlineStr">
         <is>
           <t>35260959610485000188550050001176901971337303</t>
         </is>
@@ -13420,46 +13828,55 @@
         <v>282.63</v>
       </c>
       <c r="U10" s="6" t="n">
+        <v>3374.8</v>
+      </c>
+      <c r="V10" s="6" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="W10" s="6" t="n">
+        <v>30.37</v>
+      </c>
+      <c r="X10" s="6" t="n">
         <v>3873.74</v>
       </c>
-      <c r="V10" s="5" t="inlineStr">
+      <c r="Y10" s="5" t="inlineStr">
         <is>
           <t>101 - COMPRA P/ INDUST - FORA ES</t>
         </is>
       </c>
-      <c r="W10" s="5" t="inlineStr">
+      <c r="Z10" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X10" s="6" t="n">
+      <c r="AA10" s="6" t="n">
         <v>154.95</v>
       </c>
-      <c r="Y10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA10" s="6" t="n">
+      <c r="AB10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="6" t="n">
         <v>309.9</v>
       </c>
-      <c r="AB10" s="5" t="inlineStr">
+      <c r="AE10" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506</t>
         </is>
       </c>
-      <c r="AC10" s="5" t="inlineStr">
+      <c r="AF10" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD10" s="5" t="inlineStr">
+      <c r="AG10" s="5" t="inlineStr">
         <is>
           <t>ICMS destacado (CST 00) em insumo (classificação do sped anterior); ICMS antecipado importado 8% x 3,873.74 = R$ 309.90 (E111 PR000080 débito / PR020212 crédito + E113)</t>
         </is>
       </c>
-      <c r="AE10" s="5" t="inlineStr">
+      <c r="AH10" s="5" t="inlineStr">
         <is>
           <t>35260949698723003110550550002759661838341135</t>
         </is>
@@ -13541,46 +13958,55 @@
         <v>0</v>
       </c>
       <c r="U11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="6" t="n">
         <v>948</v>
       </c>
-      <c r="V11" s="5" t="inlineStr">
+      <c r="Y11" s="5" t="inlineStr">
         <is>
           <t>144 - ENTRADA PARA IND. POR ENCO</t>
         </is>
       </c>
-      <c r="W11" s="5" t="inlineStr">
+      <c r="Z11" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z11" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB11" s="5" t="inlineStr">
+      <c r="AB11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" s="5" t="inlineStr">
         <is>
           <t>D 614 / C 607</t>
         </is>
       </c>
-      <c r="AC11" s="5" t="inlineStr">
+      <c r="AF11" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD11" s="5" t="inlineStr">
+      <c r="AG11" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por encomenda (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE11" s="5" t="inlineStr">
+      <c r="AH11" s="5" t="inlineStr">
         <is>
           <t>50260927697083000176550010000148381118293998</t>
         </is>
@@ -13662,46 +14088,55 @@
         <v>27.52</v>
       </c>
       <c r="U12" s="6" t="n">
+        <v>883.96</v>
+      </c>
+      <c r="V12" s="6" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="W12" s="6" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="X12" s="6" t="n">
         <v>1074.5</v>
       </c>
-      <c r="V12" s="5" t="inlineStr">
+      <c r="Y12" s="5" t="inlineStr">
         <is>
           <t>101 - COMPRA P/ INDUST - FORA ES</t>
         </is>
       </c>
-      <c r="W12" s="5" t="inlineStr">
+      <c r="Z12" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X12" s="6" t="n">
+      <c r="AA12" s="6" t="n">
         <v>125.11</v>
       </c>
-      <c r="Y12" s="6" t="n">
+      <c r="AB12" s="6" t="n">
         <v>31.95</v>
       </c>
-      <c r="Z12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="5" t="inlineStr">
+      <c r="AC12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506</t>
         </is>
       </c>
-      <c r="AC12" s="5" t="inlineStr">
+      <c r="AF12" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD12" s="5" t="inlineStr">
+      <c r="AG12" s="5" t="inlineStr">
         <is>
           <t>ICMS destacado (CST 00) em insumo (classificação do sped anterior)</t>
         </is>
       </c>
-      <c r="AE12" s="5" t="inlineStr">
+      <c r="AH12" s="5" t="inlineStr">
         <is>
           <t>35260918858535000163550010000482411465753374</t>
         </is>
@@ -13783,46 +14218,55 @@
         <v>352.94</v>
       </c>
       <c r="U13" s="6" t="n">
+        <v>3657.21</v>
+      </c>
+      <c r="V13" s="6" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="W13" s="6" t="n">
+        <v>32.91</v>
+      </c>
+      <c r="X13" s="6" t="n">
         <v>4794.99</v>
       </c>
-      <c r="V13" s="5" t="inlineStr">
+      <c r="Y13" s="5" t="inlineStr">
         <is>
           <t>101 - COMPRA P/ INDUST - FORA ES</t>
         </is>
       </c>
-      <c r="W13" s="5" t="inlineStr">
+      <c r="Z13" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X13" s="6" t="n">
+      <c r="AA13" s="6" t="n">
         <v>557.29</v>
       </c>
-      <c r="Y13" s="6" t="n">
+      <c r="AB13" s="6" t="n">
         <v>150.93</v>
       </c>
-      <c r="Z13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="5" t="inlineStr">
+      <c r="AC13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506</t>
         </is>
       </c>
-      <c r="AC13" s="5" t="inlineStr">
+      <c r="AF13" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD13" s="5" t="inlineStr">
+      <c r="AG13" s="5" t="inlineStr">
         <is>
           <t>ICMS destacado (CST 00) em matéria-prima (fragrância/essência)</t>
         </is>
       </c>
-      <c r="AE13" s="5" t="inlineStr">
+      <c r="AH13" s="5" t="inlineStr">
         <is>
           <t>35260962514971000107550010001418111026832844</t>
         </is>
@@ -13906,44 +14350,53 @@
       <c r="U14" s="6" t="n">
         <v>8472.040000000001</v>
       </c>
-      <c r="V14" s="5" t="inlineStr">
+      <c r="V14" s="6" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="W14" s="6" t="n">
+        <v>76.25</v>
+      </c>
+      <c r="X14" s="6" t="n">
+        <v>8472.040000000001</v>
+      </c>
+      <c r="Y14" s="5" t="inlineStr">
         <is>
           <t>155 - OUTRAS ENTRADAS DE MERCADO</t>
         </is>
       </c>
-      <c r="W14" s="5" t="inlineStr">
+      <c r="Z14" s="5" t="inlineStr">
         <is>
           <t>financeiro</t>
         </is>
       </c>
-      <c r="X14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB14" s="5" t="inlineStr">
+      <c r="AB14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="5" t="inlineStr">
         <is>
           <t>D 612 / C 613</t>
         </is>
       </c>
-      <c r="AC14" s="5" t="inlineStr">
+      <c r="AF14" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD14" s="5" t="inlineStr">
+      <c r="AG14" s="5" t="inlineStr">
         <is>
           <t>Nota sem mercadoria (antecipação/financeira)</t>
         </is>
       </c>
-      <c r="AE14" s="5" t="inlineStr">
+      <c r="AH14" s="5" t="inlineStr">
         <is>
           <t>31260958309709000820550070000003911550019201</t>
         </is>
@@ -14027,44 +14480,53 @@
       <c r="U15" s="6" t="n">
         <v>275.34</v>
       </c>
-      <c r="V15" s="5" t="inlineStr">
+      <c r="V15" s="6" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="W15" s="6" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="X15" s="6" t="n">
+        <v>275.34</v>
+      </c>
+      <c r="Y15" s="5" t="inlineStr">
         <is>
           <t>155 - OUTRAS ENTRADAS DE MERCADO</t>
         </is>
       </c>
-      <c r="W15" s="5" t="inlineStr">
+      <c r="Z15" s="5" t="inlineStr">
         <is>
           <t>financeiro</t>
         </is>
       </c>
-      <c r="X15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA15" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB15" s="5" t="inlineStr">
+      <c r="AB15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" s="5" t="inlineStr">
         <is>
           <t>D 612 / C 613</t>
         </is>
       </c>
-      <c r="AC15" s="5" t="inlineStr">
+      <c r="AF15" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD15" s="5" t="inlineStr">
+      <c r="AG15" s="5" t="inlineStr">
         <is>
           <t>Nota sem mercadoria (antecipação/financeira)</t>
         </is>
       </c>
-      <c r="AE15" s="5" t="inlineStr">
+      <c r="AH15" s="5" t="inlineStr">
         <is>
           <t>31260958309709000820550070000003921611175930</t>
         </is>
@@ -14146,46 +14608,55 @@
         <v>0</v>
       </c>
       <c r="U16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="V16" s="5" t="inlineStr">
+      <c r="Y16" s="5" t="inlineStr">
         <is>
           <t>144 - ENTRADA PARA IND. POR ENCO</t>
         </is>
       </c>
-      <c r="W16" s="5" t="inlineStr">
+      <c r="Z16" s="5" t="inlineStr">
         <is>
           <t>remessa</t>
         </is>
       </c>
-      <c r="X16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z16" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="AA16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AB16" s="5" t="inlineStr">
+      <c r="AB16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" s="5" t="inlineStr">
         <is>
           <t>D 614 / C 607</t>
         </is>
       </c>
-      <c r="AC16" s="5" t="inlineStr">
+      <c r="AF16" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD16" s="5" t="inlineStr">
+      <c r="AG16" s="5" t="inlineStr">
         <is>
           <t>Remessa para industrialização por encomenda (insumo do cliente)</t>
         </is>
       </c>
-      <c r="AE16" s="5" t="inlineStr">
+      <c r="AH16" s="5" t="inlineStr">
         <is>
           <t>50260927697083000176550010000148561118323143</t>
         </is>
@@ -14267,46 +14738,55 @@
         <v>566.61</v>
       </c>
       <c r="U17" s="6" t="n">
+        <v>6765.78</v>
+      </c>
+      <c r="V17" s="6" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="W17" s="6" t="n">
+        <v>60.89</v>
+      </c>
+      <c r="X17" s="6" t="n">
         <v>8747.379999999999</v>
       </c>
-      <c r="V17" s="5" t="inlineStr">
+      <c r="Y17" s="5" t="inlineStr">
         <is>
           <t>101 - COMPRA P/ INDUST - FORA ES</t>
         </is>
       </c>
-      <c r="W17" s="5" t="inlineStr">
+      <c r="Z17" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X17" s="6" t="n">
+      <c r="AA17" s="6" t="n">
         <v>1016.64</v>
       </c>
-      <c r="Y17" s="6" t="n">
+      <c r="AB17" s="6" t="n">
         <v>275.34</v>
       </c>
-      <c r="Z17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB17" s="5" t="inlineStr">
+      <c r="AC17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506</t>
         </is>
       </c>
-      <c r="AC17" s="5" t="inlineStr">
+      <c r="AF17" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD17" s="5" t="inlineStr">
+      <c r="AG17" s="5" t="inlineStr">
         <is>
           <t>ICMS destacado (CST 00) em matéria-prima (tensoativo)</t>
         </is>
       </c>
-      <c r="AE17" s="5" t="inlineStr">
+      <c r="AH17" s="5" t="inlineStr">
         <is>
           <t>31260958309709000820550020000193031662295529</t>
         </is>
@@ -14388,46 +14868,55 @@
         <v>115.71</v>
       </c>
       <c r="U18" s="6" t="n">
+        <v>3716.2</v>
+      </c>
+      <c r="V18" s="6" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="W18" s="6" t="n">
+        <v>33.45</v>
+      </c>
+      <c r="X18" s="6" t="n">
         <v>4278.84</v>
       </c>
-      <c r="V18" s="5" t="inlineStr">
+      <c r="Y18" s="5" t="inlineStr">
         <is>
           <t>101 - COMPRA P/ INDUST - FORA ES</t>
         </is>
       </c>
-      <c r="W18" s="5" t="inlineStr">
+      <c r="Z18" s="5" t="inlineStr">
         <is>
           <t>insumo</t>
         </is>
       </c>
-      <c r="X18" s="6" t="n">
+      <c r="AA18" s="6" t="n">
         <v>160.71</v>
       </c>
-      <c r="Y18" s="6" t="n">
+      <c r="AB18" s="6" t="n">
         <v>261.15</v>
       </c>
-      <c r="Z18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA18" s="6" t="n">
+      <c r="AC18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="6" t="n">
         <v>321.42</v>
       </c>
-      <c r="AB18" s="5" t="inlineStr">
+      <c r="AE18" s="5" t="inlineStr">
         <is>
           <t>D 56 / C 506</t>
         </is>
       </c>
-      <c r="AC18" s="5" t="inlineStr">
+      <c r="AF18" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="AD18" s="5" t="inlineStr">
+      <c r="AG18" s="5" t="inlineStr">
         <is>
           <t>ICMS destacado (CST 00) em insumo (classificação do sped anterior); ICMS antecipado importado 8% x 4,017.69 = R$ 321.42 (E111 PR000080 débito / PR020212 crédito + E113)</t>
         </is>
       </c>
-      <c r="AE18" s="5" t="inlineStr">
+      <c r="AH18" s="5" t="inlineStr">
         <is>
           <t>35260911340087000162550010000422851305252223</t>
         </is>
@@ -14498,28 +14987,40 @@
         <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*U5:U18)</f>
         <v/>
       </c>
-      <c r="V19" s="17" t="n"/>
-      <c r="W19" s="17" t="n"/>
+      <c r="V19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*V5:V18)</f>
+        <v/>
+      </c>
+      <c r="W19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*W5:W18)</f>
+        <v/>
+      </c>
       <c r="X19" s="18">
         <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*X5:X18)</f>
         <v/>
       </c>
-      <c r="Y19" s="18">
-        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*Y5:Y18)</f>
-        <v/>
-      </c>
-      <c r="Z19" s="18">
-        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*Z5:Z18)</f>
-        <v/>
-      </c>
+      <c r="Y19" s="17" t="n"/>
+      <c r="Z19" s="17" t="n"/>
       <c r="AA19" s="18">
         <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*AA5:AA18)</f>
         <v/>
       </c>
-      <c r="AB19" s="17" t="n"/>
-      <c r="AC19" s="17" t="n"/>
-      <c r="AD19" s="17" t="n"/>
+      <c r="AB19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*AB5:AB18)</f>
+        <v/>
+      </c>
+      <c r="AC19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*AC5:AC18)</f>
+        <v/>
+      </c>
+      <c r="AD19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*AD5:AD18)</f>
+        <v/>
+      </c>
       <c r="AE19" s="17" t="n"/>
+      <c r="AF19" s="17" t="n"/>
+      <c r="AG19" s="17" t="n"/>
+      <c r="AH19" s="17" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="19" t="inlineStr">
@@ -14566,7 +15067,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AE18"/>
+  <autoFilter ref="A4:AH18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Cosmetici: relações de 09/2026 com o que vai no TXT de importação (para conferência antes de importar)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpFQAF7UfcTJUBPm398Z8s
</commit_message>
<xml_diff>
--- a/Cosmetici/Fiscal/2026-09/Relacao_Entradas_Cosmetici_09-2026.xlsx
+++ b/Cosmetici/Fiscal/2026-09/Relacao_Entradas_Cosmetici_09-2026.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NFS-e tomadas" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas as entradas'!$A$4:$S$109</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NF-e dentro do estado (PR)'!$A$4:$AH$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NF-e fora do estado'!$A$4:$AH$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CT-e'!$A$4:$R$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Todas as entradas'!$A$4:$T$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NF-e dentro do estado (PR)'!$A$4:$AN$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NF-e fora do estado'!$A$4:$AN$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CT-e'!$A$4:$U$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'NFS-e tomadas'!$A$4:$AA$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S114"/>
+  <dimension ref="A1:T114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -524,8 +524,9 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="46" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="46" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -630,10 +631,15 @@
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
+          <t>Vai no TXT?</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
           <t>Observação</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>Chave</t>
         </is>
@@ -703,8 +709,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R5" s="5" t="inlineStr"/>
-      <c r="S5" s="5" t="inlineStr">
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr"/>
+      <c r="T5" s="5" t="inlineStr">
         <is>
           <t>41260906015875000143550010000037951000701710</t>
         </is>
@@ -774,8 +785,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R6" s="5" t="inlineStr"/>
-      <c r="S6" s="5" t="inlineStr">
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr"/>
+      <c r="T6" s="5" t="inlineStr">
         <is>
           <t>41260904993269000177550010000417311010503945</t>
         </is>
@@ -837,8 +853,13 @@
           <t>OK (XML sem base do ISS - Simples, sem retenção; o relatório repete o valor)</t>
         </is>
       </c>
-      <c r="R7" s="5" t="inlineStr"/>
-      <c r="S7" s="5" t="inlineStr">
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr"/>
+      <c r="T7" s="5" t="inlineStr">
         <is>
           <t>41069022207768652000110000000000154726099373367718</t>
         </is>
@@ -902,10 +923,15 @@
       </c>
       <c r="R8" s="8" t="inlineStr">
         <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S8" s="8" t="inlineStr">
+        <is>
           <t>SIM - IRRF</t>
         </is>
       </c>
-      <c r="S8" s="8" t="inlineStr">
+      <c r="T8" s="8" t="inlineStr">
         <is>
           <t>41069022267742984000157000000000001826091655988219</t>
         </is>
@@ -967,8 +993,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R9" s="5" t="inlineStr"/>
-      <c r="S9" s="5" t="inlineStr">
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr"/>
+      <c r="T9" s="5" t="inlineStr">
         <is>
           <t>41069022265649511000184000000270974726090368715311</t>
         </is>
@@ -1030,8 +1061,13 @@
           <t>OK (XML sem base do ISS - Simples, sem retenção; o relatório repete o valor)</t>
         </is>
       </c>
-      <c r="R10" s="5" t="inlineStr"/>
-      <c r="S10" s="5" t="inlineStr">
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr"/>
+      <c r="T10" s="5" t="inlineStr">
         <is>
           <t>41069022265649511000184000000270975126095154324020</t>
         </is>
@@ -1093,8 +1129,13 @@
           <t>OK (XML sem base do ISS - Simples, sem retenção; o relatório repete o valor)</t>
         </is>
       </c>
-      <c r="R11" s="5" t="inlineStr"/>
-      <c r="S11" s="5" t="inlineStr">
+      <c r="R11" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S11" s="5" t="inlineStr"/>
+      <c r="T11" s="5" t="inlineStr">
         <is>
           <t>41069022280402860000190000000000050726097638942622</t>
         </is>
@@ -1156,8 +1197,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R12" s="5" t="inlineStr"/>
-      <c r="S12" s="5" t="inlineStr">
+      <c r="R12" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr"/>
+      <c r="T12" s="5" t="inlineStr">
         <is>
           <t>41069022278738101000151000000081766026097784194236</t>
         </is>
@@ -1219,8 +1265,13 @@
           <t>OK (XML sem base do ISS - Simples, sem retenção; o relatório repete o valor)</t>
         </is>
       </c>
-      <c r="R13" s="5" t="inlineStr"/>
-      <c r="S13" s="5" t="inlineStr">
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr"/>
+      <c r="T13" s="5" t="inlineStr">
         <is>
           <t>41069022275114363000157000000000097426097081722597</t>
         </is>
@@ -1290,8 +1341,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R14" s="5" t="inlineStr"/>
-      <c r="S14" s="5" t="inlineStr">
+      <c r="R14" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="inlineStr"/>
+      <c r="T14" s="5" t="inlineStr">
         <is>
           <t>41260973636391000109550010001603261915612489</t>
         </is>
@@ -1361,8 +1417,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R15" s="5" t="inlineStr"/>
-      <c r="S15" s="5" t="inlineStr">
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr"/>
+      <c r="T15" s="5" t="inlineStr">
         <is>
           <t>41260944114040000130550010000228371000945488</t>
         </is>
@@ -1432,8 +1493,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R16" s="5" t="inlineStr"/>
-      <c r="S16" s="5" t="inlineStr">
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr"/>
+      <c r="T16" s="5" t="inlineStr">
         <is>
           <t>41260966434370000145550010000003001634619321</t>
         </is>
@@ -1503,8 +1569,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R17" s="5" t="inlineStr"/>
-      <c r="S17" s="5" t="inlineStr">
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>NÃO - sem acumulador para o CFOP de entrada</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr"/>
+      <c r="T17" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000050271834583570</t>
         </is>
@@ -1574,8 +1645,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R18" s="5" t="inlineStr"/>
-      <c r="S18" s="5" t="inlineStr">
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="inlineStr"/>
+      <c r="T18" s="5" t="inlineStr">
         <is>
           <t>41260962341566000134550010000006951857187453</t>
         </is>
@@ -1645,8 +1721,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R19" s="5" t="inlineStr"/>
-      <c r="S19" s="5" t="inlineStr">
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr"/>
+      <c r="T19" s="5" t="inlineStr">
         <is>
           <t>41260952680145000184550010000007861702940405</t>
         </is>
@@ -1714,10 +1795,15 @@
       </c>
       <c r="R20" s="11" t="inlineStr">
         <is>
+          <t>Não - cancelado (sem XML na pasta)</t>
+        </is>
+      </c>
+      <c r="S20" s="11" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S20" s="11" t="inlineStr">
+      <c r="T20" s="11" t="inlineStr">
         <is>
           <t>41260944914992003820570030046839841046839848</t>
         </is>
@@ -1785,10 +1871,15 @@
       </c>
       <c r="R21" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S21" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S21" s="14" t="inlineStr">
+      <c r="T21" s="14" t="inlineStr">
         <is>
           <t>41260944914992003820570030046879861046879869</t>
         </is>
@@ -1858,8 +1949,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R22" s="5" t="inlineStr"/>
-      <c r="S22" s="5" t="inlineStr">
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S22" s="5" t="inlineStr"/>
+      <c r="T22" s="5" t="inlineStr">
         <is>
           <t>41260941726398000125550010000049201009949200</t>
         </is>
@@ -1929,8 +2025,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R23" s="5" t="inlineStr"/>
-      <c r="S23" s="5" t="inlineStr">
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>NÃO - sem acumulador para o CFOP de entrada</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr"/>
+      <c r="T23" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000050481113690367</t>
         </is>
@@ -1992,8 +2093,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R24" s="5" t="inlineStr"/>
-      <c r="S24" s="5" t="inlineStr">
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S24" s="5" t="inlineStr"/>
+      <c r="T24" s="5" t="inlineStr">
         <is>
           <t>41069022200495545000116000000000046926091708323044</t>
         </is>
@@ -2055,8 +2161,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R25" s="5" t="inlineStr"/>
-      <c r="S25" s="5" t="inlineStr">
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr"/>
+      <c r="T25" s="5" t="inlineStr">
         <is>
           <t>41255062201790040000147000000000879826090020603825</t>
         </is>
@@ -2122,8 +2233,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R26" s="5" t="inlineStr"/>
-      <c r="S26" s="5" t="inlineStr">
+      <c r="R26" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S26" s="5" t="inlineStr"/>
+      <c r="T26" s="5" t="inlineStr">
         <is>
           <t>43260900428307000600570010055979961055979961</t>
         </is>
@@ -2193,8 +2309,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R27" s="5" t="inlineStr"/>
-      <c r="S27" s="5" t="inlineStr">
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S27" s="5" t="inlineStr"/>
+      <c r="T27" s="5" t="inlineStr">
         <is>
           <t>43260954079636000108550010000025641087230517</t>
         </is>
@@ -2256,8 +2377,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R28" s="5" t="inlineStr"/>
-      <c r="S28" s="5" t="inlineStr">
+      <c r="R28" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S28" s="5" t="inlineStr"/>
+      <c r="T28" s="5" t="inlineStr">
         <is>
           <t>35503081248395289000111000000004545426099076402305</t>
         </is>
@@ -2325,10 +2451,15 @@
       </c>
       <c r="R29" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S29" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S29" s="14" t="inlineStr">
+      <c r="T29" s="14" t="inlineStr">
         <is>
           <t>41260948740351000327570000039996291544246881</t>
         </is>
@@ -2396,10 +2527,15 @@
       </c>
       <c r="R30" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S30" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S30" s="14" t="inlineStr">
+      <c r="T30" s="14" t="inlineStr">
         <is>
           <t>41260948740351000327570000039996301101761800</t>
         </is>
@@ -2469,8 +2605,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R31" s="5" t="inlineStr"/>
-      <c r="S31" s="5" t="inlineStr">
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S31" s="5" t="inlineStr"/>
+      <c r="T31" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000050801135229929</t>
         </is>
@@ -2540,8 +2681,13 @@
           <t>Cancelada - confere: evento de cancelamento no XML e status "Cancelamento" no relatório</t>
         </is>
       </c>
-      <c r="R32" s="11" t="inlineStr"/>
-      <c r="S32" s="11" t="inlineStr">
+      <c r="R32" s="11" t="inlineStr">
+        <is>
+          <t>Sim - cancelada (situação 02)</t>
+        </is>
+      </c>
+      <c r="S32" s="11" t="inlineStr"/>
+      <c r="T32" s="11" t="inlineStr">
         <is>
           <t>41260952680145000184550010000007941049258979</t>
         </is>
@@ -2611,8 +2757,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R33" s="5" t="inlineStr"/>
-      <c r="S33" s="5" t="inlineStr">
+      <c r="R33" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S33" s="5" t="inlineStr"/>
+      <c r="T33" s="5" t="inlineStr">
         <is>
           <t>41260952680145000184550010000007951158784741</t>
         </is>
@@ -2674,8 +2825,13 @@
           <t>OK (XML sem base do ISS - Simples, sem retenção; o relatório repete o valor)</t>
         </is>
       </c>
-      <c r="R34" s="5" t="inlineStr"/>
-      <c r="S34" s="5" t="inlineStr">
+      <c r="R34" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S34" s="5" t="inlineStr"/>
+      <c r="T34" s="5" t="inlineStr">
         <is>
           <t>41069022224891333000116000000000090826090575270117</t>
         </is>
@@ -2743,10 +2899,15 @@
       </c>
       <c r="R35" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S35" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S35" s="14" t="inlineStr">
+      <c r="T35" s="14" t="inlineStr">
         <is>
           <t>35260973939449000193579990364259291604264536</t>
         </is>
@@ -2808,8 +2969,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R36" s="5" t="inlineStr"/>
-      <c r="S36" s="5" t="inlineStr">
+      <c r="R36" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S36" s="5" t="inlineStr"/>
+      <c r="T36" s="5" t="inlineStr">
         <is>
           <t>35503081232223020000118000000558882126097884718838</t>
         </is>
@@ -2879,8 +3045,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R37" s="5" t="inlineStr"/>
-      <c r="S37" s="5" t="inlineStr">
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S37" s="5" t="inlineStr"/>
+      <c r="T37" s="5" t="inlineStr">
         <is>
           <t>41260937295717000118550010000137211931581334</t>
         </is>
@@ -2950,8 +3121,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R38" s="5" t="inlineStr"/>
-      <c r="S38" s="5" t="inlineStr">
+      <c r="R38" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S38" s="5" t="inlineStr"/>
+      <c r="T38" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000051331151580428</t>
         </is>
@@ -3021,8 +3197,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R39" s="5" t="inlineStr"/>
-      <c r="S39" s="5" t="inlineStr">
+      <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S39" s="5" t="inlineStr"/>
+      <c r="T39" s="5" t="inlineStr">
         <is>
           <t>35260939237959000180550010000080991000082318</t>
         </is>
@@ -3092,8 +3273,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R40" s="5" t="inlineStr"/>
-      <c r="S40" s="5" t="inlineStr">
+      <c r="R40" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S40" s="5" t="inlineStr"/>
+      <c r="T40" s="5" t="inlineStr">
         <is>
           <t>35260934970658000148550010000081121000087609</t>
         </is>
@@ -3163,8 +3349,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R41" s="5" t="inlineStr"/>
-      <c r="S41" s="5" t="inlineStr">
+      <c r="R41" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S41" s="5" t="inlineStr"/>
+      <c r="T41" s="5" t="inlineStr">
         <is>
           <t>41260910265455000192550010000404511000405060</t>
         </is>
@@ -3234,8 +3425,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R42" s="5" t="inlineStr"/>
-      <c r="S42" s="5" t="inlineStr">
+      <c r="R42" s="5" t="inlineStr">
+        <is>
+          <t>NÃO - sem acumulador para o CFOP de entrada</t>
+        </is>
+      </c>
+      <c r="S42" s="5" t="inlineStr"/>
+      <c r="T42" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000051621201311907</t>
         </is>
@@ -3303,10 +3499,15 @@
       </c>
       <c r="R43" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S43" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S43" s="14" t="inlineStr">
+      <c r="T43" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010178175381661666021</t>
         </is>
@@ -3374,10 +3575,15 @@
       </c>
       <c r="R44" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S44" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S44" s="14" t="inlineStr">
+      <c r="T44" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010178178331686344389</t>
         </is>
@@ -3447,8 +3653,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R45" s="5" t="inlineStr"/>
-      <c r="S45" s="5" t="inlineStr">
+      <c r="R45" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S45" s="5" t="inlineStr"/>
+      <c r="T45" s="5" t="inlineStr">
         <is>
           <t>41260959087034000108550010000004181258202600</t>
         </is>
@@ -3518,8 +3729,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R46" s="5" t="inlineStr"/>
-      <c r="S46" s="5" t="inlineStr">
+      <c r="R46" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S46" s="5" t="inlineStr"/>
+      <c r="T46" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000051701177572396</t>
         </is>
@@ -3581,8 +3797,13 @@
           <t>OK (XML sem base do ISS - Simples, sem retenção; o relatório repete o valor)</t>
         </is>
       </c>
-      <c r="R47" s="5" t="inlineStr"/>
-      <c r="S47" s="5" t="inlineStr">
+      <c r="R47" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S47" s="5" t="inlineStr"/>
+      <c r="T47" s="5" t="inlineStr">
         <is>
           <t>41069022259684382000162000000000001026098158485630</t>
         </is>
@@ -3644,8 +3865,13 @@
           <t>OK (XML sem base do ISS - Simples, sem retenção; o relatório repete o valor)</t>
         </is>
       </c>
-      <c r="R48" s="5" t="inlineStr"/>
-      <c r="S48" s="5" t="inlineStr">
+      <c r="R48" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S48" s="5" t="inlineStr"/>
+      <c r="T48" s="5" t="inlineStr">
         <is>
           <t>41069022259684382000162000000000001126096345619740</t>
         </is>
@@ -3707,8 +3933,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R49" s="5" t="inlineStr"/>
-      <c r="S49" s="5" t="inlineStr">
+      <c r="R49" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S49" s="5" t="inlineStr"/>
+      <c r="T49" s="5" t="inlineStr">
         <is>
           <t>50027041214309879000162000000000953026090714785828</t>
         </is>
@@ -3776,10 +4007,15 @@
       </c>
       <c r="R50" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S50" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S50" s="14" t="inlineStr">
+      <c r="T50" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010178268311888893400</t>
         </is>
@@ -3849,8 +4085,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R51" s="5" t="inlineStr"/>
-      <c r="S51" s="5" t="inlineStr">
+      <c r="R51" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S51" s="5" t="inlineStr"/>
+      <c r="T51" s="5" t="inlineStr">
         <is>
           <t>41260944114040000130550010000231271000948452</t>
         </is>
@@ -3920,8 +4161,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R52" s="5" t="inlineStr"/>
-      <c r="S52" s="5" t="inlineStr">
+      <c r="R52" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S52" s="5" t="inlineStr"/>
+      <c r="T52" s="5" t="inlineStr">
         <is>
           <t>35260967598292000187550010000303381000323387</t>
         </is>
@@ -3991,8 +4237,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R53" s="5" t="inlineStr"/>
-      <c r="S53" s="5" t="inlineStr">
+      <c r="R53" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S53" s="5" t="inlineStr"/>
+      <c r="T53" s="5" t="inlineStr">
         <is>
           <t>41260949547438000183550010000067821963905200</t>
         </is>
@@ -4062,8 +4313,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R54" s="5" t="inlineStr"/>
-      <c r="S54" s="5" t="inlineStr">
+      <c r="R54" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S54" s="5" t="inlineStr"/>
+      <c r="T54" s="5" t="inlineStr">
         <is>
           <t>41260952680145000184550010000008141610067850</t>
         </is>
@@ -4125,8 +4381,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R55" s="5" t="inlineStr"/>
-      <c r="S55" s="5" t="inlineStr">
+      <c r="R55" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S55" s="5" t="inlineStr"/>
+      <c r="T55" s="5" t="inlineStr">
         <is>
           <t>41018041259087034000108000000000007226090000000014</t>
         </is>
@@ -4192,8 +4453,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R56" s="5" t="inlineStr"/>
-      <c r="S56" s="5" t="inlineStr">
+      <c r="R56" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S56" s="5" t="inlineStr"/>
+      <c r="T56" s="5" t="inlineStr">
         <is>
           <t>35260903867083000290570030000257091000483871</t>
         </is>
@@ -4261,10 +4527,15 @@
       </c>
       <c r="R57" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S57" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S57" s="14" t="inlineStr">
+      <c r="T57" s="14" t="inlineStr">
         <is>
           <t>41260948740351000327570000040101941868875491</t>
         </is>
@@ -4334,8 +4605,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R58" s="5" t="inlineStr"/>
-      <c r="S58" s="5" t="inlineStr">
+      <c r="R58" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S58" s="5" t="inlineStr"/>
+      <c r="T58" s="5" t="inlineStr">
         <is>
           <t>41260918074269000188550010000171871932036922</t>
         </is>
@@ -4405,8 +4681,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R59" s="5" t="inlineStr"/>
-      <c r="S59" s="5" t="inlineStr">
+      <c r="R59" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S59" s="5" t="inlineStr"/>
+      <c r="T59" s="5" t="inlineStr">
         <is>
           <t>41260925141658000144550020000032141236266620</t>
         </is>
@@ -4468,8 +4749,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R60" s="5" t="inlineStr"/>
-      <c r="S60" s="5" t="inlineStr">
+      <c r="R60" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S60" s="5" t="inlineStr"/>
+      <c r="T60" s="5" t="inlineStr">
         <is>
           <t>41069022277800407000128000000017322826095713648820</t>
         </is>
@@ -4537,10 +4823,15 @@
       </c>
       <c r="R61" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S61" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S61" s="14" t="inlineStr">
+      <c r="T61" s="14" t="inlineStr">
         <is>
           <t>41260900428307002301570010020794471020794476</t>
         </is>
@@ -4608,10 +4899,15 @@
       </c>
       <c r="R62" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S62" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S62" s="14" t="inlineStr">
+      <c r="T62" s="14" t="inlineStr">
         <is>
           <t>41260900428307002301570010020812911020812916</t>
         </is>
@@ -4679,10 +4975,15 @@
       </c>
       <c r="R63" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S63" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S63" s="14" t="inlineStr">
+      <c r="T63" s="14" t="inlineStr">
         <is>
           <t>41260900428307002301570010020812921020812921</t>
         </is>
@@ -4750,10 +5051,15 @@
       </c>
       <c r="R64" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S64" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S64" s="14" t="inlineStr">
+      <c r="T64" s="14" t="inlineStr">
         <is>
           <t>41260948740351000327570000040114621516701249</t>
         </is>
@@ -4823,8 +5129,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R65" s="5" t="inlineStr"/>
-      <c r="S65" s="5" t="inlineStr">
+      <c r="R65" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S65" s="5" t="inlineStr"/>
+      <c r="T65" s="5" t="inlineStr">
         <is>
           <t>35260959610485000188550050001176901971337303</t>
         </is>
@@ -4894,8 +5205,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R66" s="5" t="inlineStr"/>
-      <c r="S66" s="5" t="inlineStr">
+      <c r="R66" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S66" s="5" t="inlineStr"/>
+      <c r="T66" s="5" t="inlineStr">
         <is>
           <t>41260921822008000103550020000045511028307079</t>
         </is>
@@ -4965,8 +5281,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R67" s="5" t="inlineStr"/>
-      <c r="S67" s="5" t="inlineStr">
+      <c r="R67" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S67" s="5" t="inlineStr"/>
+      <c r="T67" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000052331135756040</t>
         </is>
@@ -5036,8 +5357,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R68" s="5" t="inlineStr"/>
-      <c r="S68" s="5" t="inlineStr">
+      <c r="R68" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S68" s="5" t="inlineStr"/>
+      <c r="T68" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000052351191452986</t>
         </is>
@@ -5107,8 +5433,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R69" s="5" t="inlineStr"/>
-      <c r="S69" s="5" t="inlineStr">
+      <c r="R69" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S69" s="5" t="inlineStr"/>
+      <c r="T69" s="5" t="inlineStr">
         <is>
           <t>41260906237330000181550010000558741118273450</t>
         </is>
@@ -5174,8 +5505,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R70" s="5" t="inlineStr"/>
-      <c r="S70" s="5" t="inlineStr">
+      <c r="R70" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S70" s="5" t="inlineStr"/>
+      <c r="T70" s="5" t="inlineStr">
         <is>
           <t>35260903867083000290570030000259101000487488</t>
         </is>
@@ -5245,8 +5581,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R71" s="5" t="inlineStr"/>
-      <c r="S71" s="5" t="inlineStr">
+      <c r="R71" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S71" s="5" t="inlineStr"/>
+      <c r="T71" s="5" t="inlineStr">
         <is>
           <t>35260949698723003110550550002759661838341135</t>
         </is>
@@ -5308,8 +5649,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R72" s="5" t="inlineStr"/>
-      <c r="S72" s="5" t="inlineStr">
+      <c r="R72" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S72" s="5" t="inlineStr"/>
+      <c r="T72" s="5" t="inlineStr">
         <is>
           <t>42054072204580911000196000000024307926097939111579</t>
         </is>
@@ -5371,8 +5717,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R73" s="5" t="inlineStr"/>
-      <c r="S73" s="5" t="inlineStr">
+      <c r="R73" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S73" s="5" t="inlineStr"/>
+      <c r="T73" s="5" t="inlineStr">
         <is>
           <t>41069022204523560000181000000000922726091381915688</t>
         </is>
@@ -5440,10 +5791,15 @@
       </c>
       <c r="R74" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S74" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S74" s="14" t="inlineStr">
+      <c r="T74" s="14" t="inlineStr">
         <is>
           <t>41260948740351000327570000040148961341484558</t>
         </is>
@@ -5513,8 +5869,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R75" s="5" t="inlineStr"/>
-      <c r="S75" s="5" t="inlineStr">
+      <c r="R75" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S75" s="5" t="inlineStr"/>
+      <c r="T75" s="5" t="inlineStr">
         <is>
           <t>35260962514971000107550010001418111026832844</t>
         </is>
@@ -5584,8 +5945,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R76" s="5" t="inlineStr"/>
-      <c r="S76" s="5" t="inlineStr">
+      <c r="R76" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S76" s="5" t="inlineStr"/>
+      <c r="T76" s="5" t="inlineStr">
         <is>
           <t>50260927697083000176550010000148381118293998</t>
         </is>
@@ -5655,8 +6021,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R77" s="5" t="inlineStr"/>
-      <c r="S77" s="5" t="inlineStr">
+      <c r="R77" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S77" s="5" t="inlineStr"/>
+      <c r="T77" s="5" t="inlineStr">
         <is>
           <t>35260918858535000163550010000482411465753374</t>
         </is>
@@ -5726,8 +6097,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R78" s="5" t="inlineStr"/>
-      <c r="S78" s="5" t="inlineStr">
+      <c r="R78" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S78" s="5" t="inlineStr"/>
+      <c r="T78" s="5" t="inlineStr">
         <is>
           <t>41260906237330000181550010000559131118294105</t>
         </is>
@@ -5795,10 +6171,15 @@
       </c>
       <c r="R79" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S79" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S79" s="14" t="inlineStr">
+      <c r="T79" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010178901901579809677</t>
         </is>
@@ -5866,10 +6247,15 @@
       </c>
       <c r="R80" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S80" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S80" s="14" t="inlineStr">
+      <c r="T80" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010178901911551237919</t>
         </is>
@@ -5937,10 +6323,15 @@
       </c>
       <c r="R81" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S81" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S81" s="14" t="inlineStr">
+      <c r="T81" s="14" t="inlineStr">
         <is>
           <t>41260948740351000327570000040164841595451461</t>
         </is>
@@ -6008,10 +6399,15 @@
       </c>
       <c r="R82" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S82" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S82" s="14" t="inlineStr">
+      <c r="T82" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010178962521387579519</t>
         </is>
@@ -6079,10 +6475,15 @@
       </c>
       <c r="R83" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S83" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S83" s="14" t="inlineStr">
+      <c r="T83" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179015681681992936</t>
         </is>
@@ -6150,10 +6551,15 @@
       </c>
       <c r="R84" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S84" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S84" s="14" t="inlineStr">
+      <c r="T84" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179015821611093770</t>
         </is>
@@ -6221,10 +6627,15 @@
       </c>
       <c r="R85" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S85" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S85" s="14" t="inlineStr">
+      <c r="T85" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179015831130565736</t>
         </is>
@@ -6292,10 +6703,15 @@
       </c>
       <c r="R86" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S86" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S86" s="14" t="inlineStr">
+      <c r="T86" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179015961538845580</t>
         </is>
@@ -6363,10 +6779,15 @@
       </c>
       <c r="R87" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S87" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S87" s="14" t="inlineStr">
+      <c r="T87" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179015971354021905</t>
         </is>
@@ -6434,10 +6855,15 @@
       </c>
       <c r="R88" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S88" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S88" s="14" t="inlineStr">
+      <c r="T88" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179016241104385135</t>
         </is>
@@ -6503,8 +6929,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R89" s="5" t="inlineStr"/>
-      <c r="S89" s="5" t="inlineStr">
+      <c r="R89" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S89" s="5" t="inlineStr"/>
+      <c r="T89" s="5" t="inlineStr">
         <is>
           <t>35260903867083000290570030000264111000496392</t>
         </is>
@@ -6568,10 +6999,15 @@
       </c>
       <c r="R90" s="8" t="inlineStr">
         <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S90" s="8" t="inlineStr">
+        <is>
           <t>SIM - PIS/COFINS/CSLL</t>
         </is>
       </c>
-      <c r="S90" s="8" t="inlineStr">
+      <c r="T90" s="8" t="inlineStr">
         <is>
           <t>35234042204665405000108000000000004326090442626218</t>
         </is>
@@ -6633,8 +7069,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R91" s="5" t="inlineStr"/>
-      <c r="S91" s="5" t="inlineStr">
+      <c r="R91" s="5" t="inlineStr">
+        <is>
+          <t>Não - NFS-e não entra no SPED ICMS/IPI</t>
+        </is>
+      </c>
+      <c r="S91" s="5" t="inlineStr"/>
+      <c r="T91" s="5" t="inlineStr">
         <is>
           <t>35503081232223020000118000000566135126091580598802</t>
         </is>
@@ -6702,10 +7143,15 @@
       </c>
       <c r="R92" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S92" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S92" s="14" t="inlineStr">
+      <c r="T92" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179150911045858097</t>
         </is>
@@ -6773,10 +7219,15 @@
       </c>
       <c r="R93" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S93" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S93" s="14" t="inlineStr">
+      <c r="T93" s="14" t="inlineStr">
         <is>
           <t>41260900428307002301570010020953961020953963</t>
         </is>
@@ -6846,8 +7297,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R94" s="5" t="inlineStr"/>
-      <c r="S94" s="5" t="inlineStr">
+      <c r="R94" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S94" s="5" t="inlineStr"/>
+      <c r="T94" s="5" t="inlineStr">
         <is>
           <t>31260958309709000820550070000003911550019201</t>
         </is>
@@ -6915,10 +7371,15 @@
       </c>
       <c r="R95" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S95" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S95" s="14" t="inlineStr">
+      <c r="T95" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179247371948650364</t>
         </is>
@@ -6986,10 +7447,15 @@
       </c>
       <c r="R96" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S96" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S96" s="14" t="inlineStr">
+      <c r="T96" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179248031905329170</t>
         </is>
@@ -7057,10 +7523,15 @@
       </c>
       <c r="R97" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S97" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S97" s="14" t="inlineStr">
+      <c r="T97" s="14" t="inlineStr">
         <is>
           <t>41260973939449002056570010179248111268602370</t>
         </is>
@@ -7128,10 +7599,15 @@
       </c>
       <c r="R98" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S98" s="14" t="inlineStr">
+        <is>
           <t>XML não está na pasta - dados do relatório SIEG</t>
         </is>
       </c>
-      <c r="S98" s="14" t="inlineStr">
+      <c r="T98" s="14" t="inlineStr">
         <is>
           <t>41260900428307002301570010020987981020987981</t>
         </is>
@@ -7201,8 +7677,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R99" s="5" t="inlineStr"/>
-      <c r="S99" s="5" t="inlineStr">
+      <c r="R99" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S99" s="5" t="inlineStr"/>
+      <c r="T99" s="5" t="inlineStr">
         <is>
           <t>50260927697083000176550010000148561118323143</t>
         </is>
@@ -7272,8 +7753,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R100" s="5" t="inlineStr"/>
-      <c r="S100" s="5" t="inlineStr">
+      <c r="R100" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S100" s="5" t="inlineStr"/>
+      <c r="T100" s="5" t="inlineStr">
         <is>
           <t>31260958309709000820550020000193031662295529</t>
         </is>
@@ -7343,8 +7829,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R101" s="5" t="inlineStr"/>
-      <c r="S101" s="5" t="inlineStr">
+      <c r="R101" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S101" s="5" t="inlineStr"/>
+      <c r="T101" s="5" t="inlineStr">
         <is>
           <t>41260976509488000149550010002220981017634246</t>
         </is>
@@ -7414,8 +7905,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R102" s="5" t="inlineStr"/>
-      <c r="S102" s="5" t="inlineStr">
+      <c r="R102" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S102" s="5" t="inlineStr"/>
+      <c r="T102" s="5" t="inlineStr">
         <is>
           <t>31260958309709000820550070000003921611175930</t>
         </is>
@@ -7485,8 +7981,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R103" s="5" t="inlineStr"/>
-      <c r="S103" s="5" t="inlineStr">
+      <c r="R103" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S103" s="5" t="inlineStr"/>
+      <c r="T103" s="5" t="inlineStr">
         <is>
           <t>35260911340087000162550010000422851305252223</t>
         </is>
@@ -7556,8 +8057,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R104" s="5" t="inlineStr"/>
-      <c r="S104" s="5" t="inlineStr">
+      <c r="R104" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S104" s="5" t="inlineStr"/>
+      <c r="T104" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000053821102007626</t>
         </is>
@@ -7627,8 +8133,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R105" s="5" t="inlineStr"/>
-      <c r="S105" s="5" t="inlineStr">
+      <c r="R105" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S105" s="5" t="inlineStr"/>
+      <c r="T105" s="5" t="inlineStr">
         <is>
           <t>41260906237330000181550010000560041118322920</t>
         </is>
@@ -7694,8 +8205,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R106" s="5" t="inlineStr"/>
-      <c r="S106" s="5" t="inlineStr">
+      <c r="R106" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S106" s="5" t="inlineStr"/>
+      <c r="T106" s="5" t="inlineStr">
         <is>
           <t>35260903867083000290570030000267301000504028</t>
         </is>
@@ -7765,8 +8281,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R107" s="5" t="inlineStr"/>
-      <c r="S107" s="5" t="inlineStr">
+      <c r="R107" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S107" s="5" t="inlineStr"/>
+      <c r="T107" s="5" t="inlineStr">
         <is>
           <t>41260916987597000140550010000381751288422874</t>
         </is>
@@ -7836,8 +8357,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R108" s="5" t="inlineStr"/>
-      <c r="S108" s="5" t="inlineStr">
+      <c r="R108" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S108" s="5" t="inlineStr"/>
+      <c r="T108" s="5" t="inlineStr">
         <is>
           <t>41260963460684000124550010000000421742919846</t>
         </is>
@@ -7907,8 +8433,13 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="R109" s="5" t="inlineStr"/>
-      <c r="S109" s="5" t="inlineStr">
+      <c r="R109" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S109" s="5" t="inlineStr"/>
+      <c r="T109" s="5" t="inlineStr">
         <is>
           <t>41260973419905000174550010000971451002693820</t>
         </is>
@@ -7962,6 +8493,7 @@
       <c r="Q110" s="17" t="n"/>
       <c r="R110" s="17" t="n"/>
       <c r="S110" s="17" t="n"/>
+      <c r="T110" s="17" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="19" t="inlineStr">
@@ -7997,7 +8529,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:S109"/>
+  <autoFilter ref="A4:T109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -8009,7 +8541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH40"/>
+  <dimension ref="A1:AN40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8045,7 +8577,13 @@
     <col width="14" customWidth="1" min="31" max="31"/>
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="50" customWidth="1" min="33" max="33"/>
-    <col width="46" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="34" max="34"/>
+    <col width="11" customWidth="1" min="35" max="35"/>
+    <col width="10" customWidth="1" min="36" max="36"/>
+    <col width="9" customWidth="1" min="37" max="37"/>
+    <col width="8" customWidth="1" min="38" max="38"/>
+    <col width="9" customWidth="1" min="39" max="39"/>
+    <col width="46" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8230,6 +8768,36 @@
       </c>
       <c r="AH4" s="3" t="inlineStr">
         <is>
+          <t>Vai no TXT?</t>
+        </is>
+      </c>
+      <c r="AI4" s="3" t="inlineStr">
+        <is>
+          <t>Base ICMS no TXT</t>
+        </is>
+      </c>
+      <c r="AJ4" s="3" t="inlineStr">
+        <is>
+          <t>ICMS no TXT</t>
+        </is>
+      </c>
+      <c r="AK4" s="3" t="inlineStr">
+        <is>
+          <t>IPI no TXT</t>
+        </is>
+      </c>
+      <c r="AL4" s="3" t="inlineStr">
+        <is>
+          <t>PIS no TXT</t>
+        </is>
+      </c>
+      <c r="AM4" s="3" t="inlineStr">
+        <is>
+          <t>COFINS no TXT</t>
+        </is>
+      </c>
+      <c r="AN4" s="3" t="inlineStr">
+        <is>
           <t>Chave de acesso</t>
         </is>
       </c>
@@ -8360,6 +8928,26 @@
       </c>
       <c r="AH5" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN5" s="5" t="inlineStr">
+        <is>
           <t>41260906015875000143550010000037951000701710</t>
         </is>
       </c>
@@ -8490,6 +9078,26 @@
       </c>
       <c r="AH6" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI6" s="6" t="n">
+        <v>1870</v>
+      </c>
+      <c r="AJ6" s="6" t="n">
+        <v>224.41</v>
+      </c>
+      <c r="AK6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="6" t="n">
+        <v>27.15</v>
+      </c>
+      <c r="AM6" s="6" t="n">
+        <v>125.06</v>
+      </c>
+      <c r="AN6" s="5" t="inlineStr">
+        <is>
           <t>41260904993269000177550010000417311010503945</t>
         </is>
       </c>
@@ -8620,6 +9228,26 @@
       </c>
       <c r="AH7" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN7" s="5" t="inlineStr">
+        <is>
           <t>41260966434370000145550010000003001634619321</t>
         </is>
       </c>
@@ -8750,6 +9378,26 @@
       </c>
       <c r="AH8" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN8" s="5" t="inlineStr">
+        <is>
           <t>41260962341566000134550010000006951857187453</t>
         </is>
       </c>
@@ -8880,6 +9528,26 @@
       </c>
       <c r="AH9" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" s="5" t="inlineStr">
+        <is>
           <t>41260952680145000184550010000007861702940405</t>
         </is>
       </c>
@@ -9010,6 +9678,16 @@
       </c>
       <c r="AH10" s="5" t="inlineStr">
         <is>
+          <t>NÃO - sem acumulador para o CFOP de entrada</t>
+        </is>
+      </c>
+      <c r="AI10" s="6" t="n"/>
+      <c r="AJ10" s="6" t="n"/>
+      <c r="AK10" s="6" t="n"/>
+      <c r="AL10" s="6" t="n"/>
+      <c r="AM10" s="6" t="n"/>
+      <c r="AN10" s="5" t="inlineStr">
+        <is>
           <t>41260903839251000152550030000050271834583570</t>
         </is>
       </c>
@@ -9140,6 +9818,26 @@
       </c>
       <c r="AH11" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI11" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ11" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AK11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN11" s="5" t="inlineStr">
+        <is>
           <t>41260944114040000130550010000228371000945488</t>
         </is>
       </c>
@@ -9270,6 +9968,26 @@
       </c>
       <c r="AH12" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN12" s="5" t="inlineStr">
+        <is>
           <t>41260973636391000109550010001603261915612489</t>
         </is>
       </c>
@@ -9400,6 +10118,26 @@
       </c>
       <c r="AH13" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN13" s="5" t="inlineStr">
+        <is>
           <t>41260941726398000125550010000049201009949200</t>
         </is>
       </c>
@@ -9529,6 +10267,16 @@
         </is>
       </c>
       <c r="AH14" s="5" t="inlineStr">
+        <is>
+          <t>NÃO - sem acumulador para o CFOP de entrada</t>
+        </is>
+      </c>
+      <c r="AI14" s="6" t="n"/>
+      <c r="AJ14" s="6" t="n"/>
+      <c r="AK14" s="6" t="n"/>
+      <c r="AL14" s="6" t="n"/>
+      <c r="AM14" s="6" t="n"/>
+      <c r="AN14" s="5" t="inlineStr">
         <is>
           <t>41260903839251000152550030000050481113690367</t>
         </is>
@@ -9640,6 +10388,16 @@
       <c r="AG15" s="11" t="inlineStr"/>
       <c r="AH15" s="11" t="inlineStr">
         <is>
+          <t>Sim - cancelada (situação 02)</t>
+        </is>
+      </c>
+      <c r="AI15" s="12" t="n"/>
+      <c r="AJ15" s="12" t="n"/>
+      <c r="AK15" s="12" t="n"/>
+      <c r="AL15" s="12" t="n"/>
+      <c r="AM15" s="12" t="n"/>
+      <c r="AN15" s="11" t="inlineStr">
+        <is>
           <t>41260952680145000184550010000007941049258979</t>
         </is>
       </c>
@@ -9770,6 +10528,26 @@
       </c>
       <c r="AH16" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN16" s="5" t="inlineStr">
+        <is>
           <t>41260952680145000184550010000007951158784741</t>
         </is>
       </c>
@@ -9900,6 +10678,26 @@
       </c>
       <c r="AH17" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN17" s="5" t="inlineStr">
+        <is>
           <t>41260903839251000152550030000050801135229929</t>
         </is>
       </c>
@@ -10030,6 +10828,26 @@
       </c>
       <c r="AH18" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN18" s="5" t="inlineStr">
+        <is>
           <t>41260903839251000152550030000051331151580428</t>
         </is>
       </c>
@@ -10160,6 +10978,26 @@
       </c>
       <c r="AH19" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN19" s="5" t="inlineStr">
+        <is>
           <t>41260937295717000118550010000137211931581334</t>
         </is>
       </c>
@@ -10290,6 +11128,16 @@
       </c>
       <c r="AH20" s="5" t="inlineStr">
         <is>
+          <t>NÃO - sem acumulador para o CFOP de entrada</t>
+        </is>
+      </c>
+      <c r="AI20" s="6" t="n"/>
+      <c r="AJ20" s="6" t="n"/>
+      <c r="AK20" s="6" t="n"/>
+      <c r="AL20" s="6" t="n"/>
+      <c r="AM20" s="6" t="n"/>
+      <c r="AN20" s="5" t="inlineStr">
+        <is>
           <t>41260903839251000152550030000051621201311907</t>
         </is>
       </c>
@@ -10420,6 +11268,26 @@
       </c>
       <c r="AH21" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN21" s="5" t="inlineStr">
+        <is>
           <t>41260910265455000192550010000404511000405060</t>
         </is>
       </c>
@@ -10550,6 +11418,26 @@
       </c>
       <c r="AH22" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN22" s="5" t="inlineStr">
+        <is>
           <t>41260959087034000108550010000004181258202600</t>
         </is>
       </c>
@@ -10680,6 +11568,26 @@
       </c>
       <c r="AH23" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN23" s="5" t="inlineStr">
+        <is>
           <t>41260903839251000152550030000051701177572396</t>
         </is>
       </c>
@@ -10810,6 +11718,26 @@
       </c>
       <c r="AH24" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN24" s="5" t="inlineStr">
+        <is>
           <t>41260952680145000184550010000008141610067850</t>
         </is>
       </c>
@@ -10940,6 +11868,26 @@
       </c>
       <c r="AH25" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN25" s="5" t="inlineStr">
+        <is>
           <t>41260949547438000183550010000067821963905200</t>
         </is>
       </c>
@@ -11070,6 +12018,26 @@
       </c>
       <c r="AH26" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ26" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AK26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN26" s="5" t="inlineStr">
+        <is>
           <t>41260944114040000130550010000231271000948452</t>
         </is>
       </c>
@@ -11200,6 +12168,26 @@
       </c>
       <c r="AH27" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN27" s="5" t="inlineStr">
+        <is>
           <t>41260925141658000144550020000032141236266620</t>
         </is>
       </c>
@@ -11330,6 +12318,26 @@
       </c>
       <c r="AH28" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN28" s="5" t="inlineStr">
+        <is>
           <t>41260918074269000188550010000171871932036922</t>
         </is>
       </c>
@@ -11460,6 +12468,26 @@
       </c>
       <c r="AH29" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN29" s="5" t="inlineStr">
+        <is>
           <t>41260921822008000103550020000045511028307079</t>
         </is>
       </c>
@@ -11590,6 +12618,26 @@
       </c>
       <c r="AH30" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN30" s="5" t="inlineStr">
+        <is>
           <t>41260903839251000152550030000052331135756040</t>
         </is>
       </c>
@@ -11720,6 +12768,26 @@
       </c>
       <c r="AH31" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN31" s="5" t="inlineStr">
+        <is>
           <t>41260903839251000152550030000052351191452986</t>
         </is>
       </c>
@@ -11850,6 +12918,26 @@
       </c>
       <c r="AH32" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN32" s="5" t="inlineStr">
+        <is>
           <t>41260906237330000181550010000558741118273450</t>
         </is>
       </c>
@@ -11980,6 +13068,26 @@
       </c>
       <c r="AH33" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN33" s="5" t="inlineStr">
+        <is>
           <t>41260906237330000181550010000559131118294105</t>
         </is>
       </c>
@@ -12110,6 +13218,26 @@
       </c>
       <c r="AH34" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN34" s="5" t="inlineStr">
+        <is>
           <t>41260903839251000152550030000053821102007626</t>
         </is>
       </c>
@@ -12240,6 +13368,26 @@
       </c>
       <c r="AH35" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN35" s="5" t="inlineStr">
+        <is>
           <t>41260906237330000181550010000560041118322920</t>
         </is>
       </c>
@@ -12370,6 +13518,26 @@
       </c>
       <c r="AH36" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN36" s="5" t="inlineStr">
+        <is>
           <t>41260976509488000149550010002220981017634246</t>
         </is>
       </c>
@@ -12500,6 +13668,26 @@
       </c>
       <c r="AH37" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN37" s="5" t="inlineStr">
+        <is>
           <t>41260963460684000124550010000000421742919846</t>
         </is>
       </c>
@@ -12630,6 +13818,26 @@
       </c>
       <c r="AH38" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI38" s="6" t="n">
+        <v>5593.5</v>
+      </c>
+      <c r="AJ38" s="6" t="n">
+        <v>671.22</v>
+      </c>
+      <c r="AK38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL38" s="6" t="n">
+        <v>81.22</v>
+      </c>
+      <c r="AM38" s="6" t="n">
+        <v>374.09</v>
+      </c>
+      <c r="AN38" s="5" t="inlineStr">
+        <is>
           <t>41260916987597000140550010000381751288422874</t>
         </is>
       </c>
@@ -12759,6 +13967,26 @@
         </is>
       </c>
       <c r="AH39" s="5" t="inlineStr">
+        <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN39" s="5" t="inlineStr">
         <is>
           <t>41260973419905000174550010000971451002693820</t>
         </is>
@@ -12863,9 +14091,30 @@
       <c r="AF40" s="17" t="n"/>
       <c r="AG40" s="17" t="n"/>
       <c r="AH40" s="17" t="n"/>
+      <c r="AI40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*AI5:AI39)</f>
+        <v/>
+      </c>
+      <c r="AJ40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*AJ5:AJ39)</f>
+        <v/>
+      </c>
+      <c r="AK40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*AK5:AK39)</f>
+        <v/>
+      </c>
+      <c r="AL40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*AL5:AL39)</f>
+        <v/>
+      </c>
+      <c r="AM40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*AM5:AM39)</f>
+        <v/>
+      </c>
+      <c r="AN40" s="17" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AH39"/>
+  <autoFilter ref="A4:AN39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -12877,7 +14126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH24"/>
+  <dimension ref="A1:AN24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12913,7 +14162,13 @@
     <col width="14" customWidth="1" min="31" max="31"/>
     <col width="26" customWidth="1" min="32" max="32"/>
     <col width="50" customWidth="1" min="33" max="33"/>
-    <col width="46" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="34" max="34"/>
+    <col width="11" customWidth="1" min="35" max="35"/>
+    <col width="10" customWidth="1" min="36" max="36"/>
+    <col width="9" customWidth="1" min="37" max="37"/>
+    <col width="8" customWidth="1" min="38" max="38"/>
+    <col width="9" customWidth="1" min="39" max="39"/>
+    <col width="46" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13098,6 +14353,36 @@
       </c>
       <c r="AH4" s="3" t="inlineStr">
         <is>
+          <t>Vai no TXT?</t>
+        </is>
+      </c>
+      <c r="AI4" s="3" t="inlineStr">
+        <is>
+          <t>Base ICMS no TXT</t>
+        </is>
+      </c>
+      <c r="AJ4" s="3" t="inlineStr">
+        <is>
+          <t>ICMS no TXT</t>
+        </is>
+      </c>
+      <c r="AK4" s="3" t="inlineStr">
+        <is>
+          <t>IPI no TXT</t>
+        </is>
+      </c>
+      <c r="AL4" s="3" t="inlineStr">
+        <is>
+          <t>PIS no TXT</t>
+        </is>
+      </c>
+      <c r="AM4" s="3" t="inlineStr">
+        <is>
+          <t>COFINS no TXT</t>
+        </is>
+      </c>
+      <c r="AN4" s="3" t="inlineStr">
+        <is>
           <t>Chave de acesso</t>
         </is>
       </c>
@@ -13228,6 +14513,26 @@
       </c>
       <c r="AH5" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="AI5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN5" s="5" t="inlineStr">
+        <is>
           <t>43260954079636000108550010000025641087230517</t>
         </is>
       </c>
@@ -13358,6 +14663,26 @@
       </c>
       <c r="AH6" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN6" s="5" t="inlineStr">
+        <is>
           <t>35260939237959000180550010000080991000082318</t>
         </is>
       </c>
@@ -13488,6 +14813,26 @@
       </c>
       <c r="AH7" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN7" s="5" t="inlineStr">
+        <is>
           <t>35260934970658000148550010000081121000087609</t>
         </is>
       </c>
@@ -13618,6 +14963,26 @@
       </c>
       <c r="AH8" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI8" s="6" t="n">
+        <v>2506.56</v>
+      </c>
+      <c r="AJ8" s="6" t="n">
+        <v>300.79</v>
+      </c>
+      <c r="AK8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" s="6" t="n">
+        <v>14.34</v>
+      </c>
+      <c r="AM8" s="6" t="n">
+        <v>66.17</v>
+      </c>
+      <c r="AN8" s="5" t="inlineStr">
+        <is>
           <t>35260967598292000187550010000303381000323387</t>
         </is>
       </c>
@@ -13748,6 +15113,26 @@
       </c>
       <c r="AH9" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI9" s="6" t="n">
+        <v>24897.18</v>
+      </c>
+      <c r="AJ9" s="6" t="n">
+        <v>2987.66</v>
+      </c>
+      <c r="AK9" s="6" t="n">
+        <v>1618.32</v>
+      </c>
+      <c r="AL9" s="6" t="n">
+        <v>361.51</v>
+      </c>
+      <c r="AM9" s="6" t="n">
+        <v>1665.12</v>
+      </c>
+      <c r="AN9" s="5" t="inlineStr">
+        <is>
           <t>35260959610485000188550050001176901971337303</t>
         </is>
       </c>
@@ -13878,6 +15263,26 @@
       </c>
       <c r="AH10" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI10" s="6" t="n">
+        <v>3873.74</v>
+      </c>
+      <c r="AJ10" s="6" t="n">
+        <v>154.95</v>
+      </c>
+      <c r="AK10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" s="6" t="n">
+        <v>61.36</v>
+      </c>
+      <c r="AM10" s="6" t="n">
+        <v>282.63</v>
+      </c>
+      <c r="AN10" s="5" t="inlineStr">
+        <is>
           <t>35260949698723003110550550002759661838341135</t>
         </is>
       </c>
@@ -14008,6 +15413,26 @@
       </c>
       <c r="AH11" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN11" s="5" t="inlineStr">
+        <is>
           <t>50260927697083000176550010000148381118293998</t>
         </is>
       </c>
@@ -14138,6 +15563,26 @@
       </c>
       <c r="AH12" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI12" s="6" t="n">
+        <v>1042.55</v>
+      </c>
+      <c r="AJ12" s="6" t="n">
+        <v>125.11</v>
+      </c>
+      <c r="AK12" s="6" t="n">
+        <v>31.95</v>
+      </c>
+      <c r="AL12" s="6" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="AM12" s="6" t="n">
+        <v>27.52</v>
+      </c>
+      <c r="AN12" s="5" t="inlineStr">
+        <is>
           <t>35260918858535000163550010000482411465753374</t>
         </is>
       </c>
@@ -14268,6 +15713,26 @@
       </c>
       <c r="AH13" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI13" s="6" t="n">
+        <v>4644.06</v>
+      </c>
+      <c r="AJ13" s="6" t="n">
+        <v>557.29</v>
+      </c>
+      <c r="AK13" s="6" t="n">
+        <v>150.93</v>
+      </c>
+      <c r="AL13" s="6" t="n">
+        <v>76.62</v>
+      </c>
+      <c r="AM13" s="6" t="n">
+        <v>352.94</v>
+      </c>
+      <c r="AN13" s="5" t="inlineStr">
+        <is>
           <t>35260962514971000107550010001418111026832844</t>
         </is>
       </c>
@@ -14398,6 +15863,26 @@
       </c>
       <c r="AH14" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN14" s="5" t="inlineStr">
+        <is>
           <t>31260958309709000820550070000003911550019201</t>
         </is>
       </c>
@@ -14528,6 +16013,26 @@
       </c>
       <c r="AH15" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN15" s="5" t="inlineStr">
+        <is>
           <t>31260958309709000820550070000003921611175930</t>
         </is>
       </c>
@@ -14658,6 +16163,26 @@
       </c>
       <c r="AH16" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN16" s="5" t="inlineStr">
+        <is>
           <t>50260927697083000176550010000148561118323143</t>
         </is>
       </c>
@@ -14788,6 +16313,26 @@
       </c>
       <c r="AH17" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI17" s="6" t="n">
+        <v>8472.040000000001</v>
+      </c>
+      <c r="AJ17" s="6" t="n">
+        <v>1016.64</v>
+      </c>
+      <c r="AK17" s="6" t="n">
+        <v>275.34</v>
+      </c>
+      <c r="AL17" s="6" t="n">
+        <v>123.01</v>
+      </c>
+      <c r="AM17" s="6" t="n">
+        <v>566.61</v>
+      </c>
+      <c r="AN17" s="5" t="inlineStr">
+        <is>
           <t>31260958309709000820550020000193031662295529</t>
         </is>
       </c>
@@ -14917,6 +16462,26 @@
         </is>
       </c>
       <c r="AH18" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="AI18" s="6" t="n">
+        <v>4017.69</v>
+      </c>
+      <c r="AJ18" s="6" t="n">
+        <v>160.71</v>
+      </c>
+      <c r="AK18" s="6" t="n">
+        <v>261.15</v>
+      </c>
+      <c r="AL18" s="6" t="n">
+        <v>25.07</v>
+      </c>
+      <c r="AM18" s="6" t="n">
+        <v>115.71</v>
+      </c>
+      <c r="AN18" s="5" t="inlineStr">
         <is>
           <t>35260911340087000162550010000422851305252223</t>
         </is>
@@ -15021,6 +16586,27 @@
       <c r="AF19" s="17" t="n"/>
       <c r="AG19" s="17" t="n"/>
       <c r="AH19" s="17" t="n"/>
+      <c r="AI19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*AI5:AI18)</f>
+        <v/>
+      </c>
+      <c r="AJ19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*AJ5:AJ18)</f>
+        <v/>
+      </c>
+      <c r="AK19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*AK5:AK18)</f>
+        <v/>
+      </c>
+      <c r="AL19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*AL5:AL18)</f>
+        <v/>
+      </c>
+      <c r="AM19" s="18">
+        <f>SUMPRODUCT((G5:G18&lt;&gt;"Cancelada")*(G5:G18&lt;&gt;"Cancelado")*AM5:AM18)</f>
+        <v/>
+      </c>
+      <c r="AN19" s="17" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="19" t="inlineStr">
@@ -15067,7 +16653,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AH18"/>
+  <autoFilter ref="A4:AN18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -15079,7 +16665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -15099,7 +16685,10 @@
     <col width="26" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="30" customWidth="1" min="17" max="17"/>
-    <col width="46" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="46" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15204,6 +16793,21 @@
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
+          <t>Vai no TXT?</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>Base ICMS no TXT</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>ICMS no TXT</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
           <t>Chave de acesso</t>
         </is>
       </c>
@@ -15284,6 +16888,13 @@
       </c>
       <c r="R5" s="11" t="inlineStr">
         <is>
+          <t>Não - cancelado (sem XML na pasta)</t>
+        </is>
+      </c>
+      <c r="S5" s="12" t="n"/>
+      <c r="T5" s="12" t="n"/>
+      <c r="U5" s="11" t="inlineStr">
+        <is>
           <t>41260944914992003820570030046839841046839848</t>
         </is>
       </c>
@@ -15364,6 +16975,13 @@
       </c>
       <c r="R6" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S6" s="15" t="n"/>
+      <c r="T6" s="15" t="n"/>
+      <c r="U6" s="14" t="inlineStr">
+        <is>
           <t>41260944914992003820570030046879861046879869</t>
         </is>
       </c>
@@ -15444,6 +17062,17 @@
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
+          <t>Sim - uso e consumo: bases zeradas</t>
+        </is>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
           <t>43260900428307000600570010055979961055979961</t>
         </is>
       </c>
@@ -15524,6 +17153,13 @@
       </c>
       <c r="R8" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S8" s="15" t="n"/>
+      <c r="T8" s="15" t="n"/>
+      <c r="U8" s="14" t="inlineStr">
+        <is>
           <t>41260948740351000327570000039996291544246881</t>
         </is>
       </c>
@@ -15604,6 +17240,13 @@
       </c>
       <c r="R9" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S9" s="15" t="n"/>
+      <c r="T9" s="15" t="n"/>
+      <c r="U9" s="14" t="inlineStr">
+        <is>
           <t>41260948740351000327570000039996301101761800</t>
         </is>
       </c>
@@ -15684,6 +17327,13 @@
       </c>
       <c r="R10" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S10" s="15" t="n"/>
+      <c r="T10" s="15" t="n"/>
+      <c r="U10" s="14" t="inlineStr">
+        <is>
           <t>35260973939449000193579990364259291604264536</t>
         </is>
       </c>
@@ -15764,6 +17414,13 @@
       </c>
       <c r="R11" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S11" s="15" t="n"/>
+      <c r="T11" s="15" t="n"/>
+      <c r="U11" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010178175381661666021</t>
         </is>
       </c>
@@ -15844,6 +17501,13 @@
       </c>
       <c r="R12" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S12" s="15" t="n"/>
+      <c r="T12" s="15" t="n"/>
+      <c r="U12" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010178178331686344389</t>
         </is>
       </c>
@@ -15924,6 +17588,13 @@
       </c>
       <c r="R13" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S13" s="15" t="n"/>
+      <c r="T13" s="15" t="n"/>
+      <c r="U13" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010178268311888893400</t>
         </is>
       </c>
@@ -16004,6 +17675,17 @@
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S14" s="6" t="n">
+        <v>116.03</v>
+      </c>
+      <c r="T14" s="6" t="n">
+        <v>13.92</v>
+      </c>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
           <t>35260903867083000290570030000257091000483871</t>
         </is>
       </c>
@@ -16084,6 +17766,13 @@
       </c>
       <c r="R15" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S15" s="15" t="n"/>
+      <c r="T15" s="15" t="n"/>
+      <c r="U15" s="14" t="inlineStr">
+        <is>
           <t>41260948740351000327570000040101941868875491</t>
         </is>
       </c>
@@ -16164,6 +17853,13 @@
       </c>
       <c r="R16" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S16" s="15" t="n"/>
+      <c r="T16" s="15" t="n"/>
+      <c r="U16" s="14" t="inlineStr">
+        <is>
           <t>41260900428307002301570010020794471020794476</t>
         </is>
       </c>
@@ -16244,6 +17940,13 @@
       </c>
       <c r="R17" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S17" s="15" t="n"/>
+      <c r="T17" s="15" t="n"/>
+      <c r="U17" s="14" t="inlineStr">
+        <is>
           <t>41260900428307002301570010020812911020812916</t>
         </is>
       </c>
@@ -16324,6 +18027,13 @@
       </c>
       <c r="R18" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S18" s="15" t="n"/>
+      <c r="T18" s="15" t="n"/>
+      <c r="U18" s="14" t="inlineStr">
+        <is>
           <t>41260900428307002301570010020812921020812921</t>
         </is>
       </c>
@@ -16404,6 +18114,13 @@
       </c>
       <c r="R19" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S19" s="15" t="n"/>
+      <c r="T19" s="15" t="n"/>
+      <c r="U19" s="14" t="inlineStr">
+        <is>
           <t>41260948740351000327570000040114621516701249</t>
         </is>
       </c>
@@ -16484,6 +18201,17 @@
       </c>
       <c r="R20" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S20" s="6" t="n">
+        <v>812.3</v>
+      </c>
+      <c r="T20" s="6" t="n">
+        <v>97.48</v>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
           <t>35260903867083000290570030000259101000487488</t>
         </is>
       </c>
@@ -16564,6 +18292,13 @@
       </c>
       <c r="R21" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S21" s="15" t="n"/>
+      <c r="T21" s="15" t="n"/>
+      <c r="U21" s="14" t="inlineStr">
+        <is>
           <t>41260948740351000327570000040148961341484558</t>
         </is>
       </c>
@@ -16644,6 +18379,13 @@
       </c>
       <c r="R22" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S22" s="15" t="n"/>
+      <c r="T22" s="15" t="n"/>
+      <c r="U22" s="14" t="inlineStr">
+        <is>
           <t>41260948740351000327570000040164841595451461</t>
         </is>
       </c>
@@ -16724,6 +18466,13 @@
       </c>
       <c r="R23" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S23" s="15" t="n"/>
+      <c r="T23" s="15" t="n"/>
+      <c r="U23" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010178901901579809677</t>
         </is>
       </c>
@@ -16804,6 +18553,13 @@
       </c>
       <c r="R24" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S24" s="15" t="n"/>
+      <c r="T24" s="15" t="n"/>
+      <c r="U24" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010178901911551237919</t>
         </is>
       </c>
@@ -16884,6 +18640,17 @@
       </c>
       <c r="R25" s="5" t="inlineStr">
         <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S25" s="6" t="n">
+        <v>126.02</v>
+      </c>
+      <c r="T25" s="6" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="U25" s="5" t="inlineStr">
+        <is>
           <t>35260903867083000290570030000264111000496392</t>
         </is>
       </c>
@@ -16964,6 +18731,13 @@
       </c>
       <c r="R26" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S26" s="15" t="n"/>
+      <c r="T26" s="15" t="n"/>
+      <c r="U26" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010178962521387579519</t>
         </is>
       </c>
@@ -17044,6 +18818,13 @@
       </c>
       <c r="R27" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S27" s="15" t="n"/>
+      <c r="T27" s="15" t="n"/>
+      <c r="U27" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179015681681992936</t>
         </is>
       </c>
@@ -17124,6 +18905,13 @@
       </c>
       <c r="R28" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S28" s="15" t="n"/>
+      <c r="T28" s="15" t="n"/>
+      <c r="U28" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179015821611093770</t>
         </is>
       </c>
@@ -17204,6 +18992,13 @@
       </c>
       <c r="R29" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S29" s="15" t="n"/>
+      <c r="T29" s="15" t="n"/>
+      <c r="U29" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179015831130565736</t>
         </is>
       </c>
@@ -17284,6 +19079,13 @@
       </c>
       <c r="R30" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S30" s="15" t="n"/>
+      <c r="T30" s="15" t="n"/>
+      <c r="U30" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179015961538845580</t>
         </is>
       </c>
@@ -17364,6 +19166,13 @@
       </c>
       <c r="R31" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S31" s="15" t="n"/>
+      <c r="T31" s="15" t="n"/>
+      <c r="U31" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179015971354021905</t>
         </is>
       </c>
@@ -17444,6 +19253,13 @@
       </c>
       <c r="R32" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S32" s="15" t="n"/>
+      <c r="T32" s="15" t="n"/>
+      <c r="U32" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179016241104385135</t>
         </is>
       </c>
@@ -17524,6 +19340,13 @@
       </c>
       <c r="R33" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S33" s="15" t="n"/>
+      <c r="T33" s="15" t="n"/>
+      <c r="U33" s="14" t="inlineStr">
+        <is>
           <t>41260900428307002301570010020953961020953963</t>
         </is>
       </c>
@@ -17604,6 +19427,13 @@
       </c>
       <c r="R34" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S34" s="15" t="n"/>
+      <c r="T34" s="15" t="n"/>
+      <c r="U34" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179150911045858097</t>
         </is>
       </c>
@@ -17684,6 +19514,13 @@
       </c>
       <c r="R35" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S35" s="15" t="n"/>
+      <c r="T35" s="15" t="n"/>
+      <c r="U35" s="14" t="inlineStr">
+        <is>
           <t>41260900428307002301570010020987981020987981</t>
         </is>
       </c>
@@ -17764,6 +19601,13 @@
       </c>
       <c r="R36" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S36" s="15" t="n"/>
+      <c r="T36" s="15" t="n"/>
+      <c r="U36" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179247371948650364</t>
         </is>
       </c>
@@ -17844,6 +19688,13 @@
       </c>
       <c r="R37" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S37" s="15" t="n"/>
+      <c r="T37" s="15" t="n"/>
+      <c r="U37" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179248031905329170</t>
         </is>
       </c>
@@ -17924,6 +19775,13 @@
       </c>
       <c r="R38" s="14" t="inlineStr">
         <is>
+          <t>NÃO - sem XML na pasta (pedir o XML)</t>
+        </is>
+      </c>
+      <c r="S38" s="15" t="n"/>
+      <c r="T38" s="15" t="n"/>
+      <c r="U38" s="14" t="inlineStr">
+        <is>
           <t>41260973939449002056570010179248111268602370</t>
         </is>
       </c>
@@ -18003,6 +19861,17 @@
         </is>
       </c>
       <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>Sim - exatamente o XML</t>
+        </is>
+      </c>
+      <c r="S39" s="6" t="n">
+        <v>188.49</v>
+      </c>
+      <c r="T39" s="6" t="n">
+        <v>22.62</v>
+      </c>
+      <c r="U39" s="5" t="inlineStr">
         <is>
           <t>35260903867083000290570030000267301000504028</t>
         </is>
@@ -18043,6 +19912,15 @@
       <c r="P40" s="17" t="n"/>
       <c r="Q40" s="17" t="n"/>
       <c r="R40" s="17" t="n"/>
+      <c r="S40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*S5:S39)</f>
+        <v/>
+      </c>
+      <c r="T40" s="18">
+        <f>SUMPRODUCT((G5:G39&lt;&gt;"Cancelada")*(G5:G39&lt;&gt;"Cancelado")*T5:T39)</f>
+        <v/>
+      </c>
+      <c r="U40" s="17" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="19" t="inlineStr">
@@ -18089,7 +19967,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:R39"/>
+  <autoFilter ref="A4:U39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Cosmetici: crédito do Simples (CSOSN 101 com vCredICMSSN, atividade-fim) no TXT de importação
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpFQAF7UfcTJUBPm398Z8s
</commit_message>
<xml_diff>
--- a/Cosmetici/Fiscal/2026-09/Relacao_Entradas_Cosmetici_09-2026.xlsx
+++ b/Cosmetici/Fiscal/2026-09/Relacao_Entradas_Cosmetici_09-2026.xlsx
@@ -9460,10 +9460,10 @@
         </is>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0</v>
+        <v>3460</v>
       </c>
       <c r="AJ5" s="6" t="n">
-        <v>0</v>
+        <v>98.95</v>
       </c>
       <c r="AK5" s="6" t="n">
         <v>0</v>

</xml_diff>